<commit_message>
Updated excel sheets for practitioner and practitionerRole
</commit_message>
<xml_diff>
--- a/input/requirements/Practitioner.xlsx
+++ b/input/requirements/Practitioner.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Practitioner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2640" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CDEA821-C0CA-443C-AA04-55A75BC67655}"/>
+  <xr:revisionPtr revIDLastSave="2665" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EEB638E-5AF9-404D-A5E8-B4AC8CB6DD37}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="655" firstSheet="3" activeTab="2" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="655" firstSheet="2" activeTab="4" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Context" sheetId="3" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="147">
   <si>
     <t>Veld</t>
   </si>
@@ -321,90 +321,90 @@
     <t>Zib 2020</t>
   </si>
   <si>
+    <t>zib2020</t>
+  </si>
+  <si>
+    <t>ZVL-002</t>
+  </si>
+  <si>
+    <t>Naamgegevens</t>
+  </si>
+  <si>
+    <t>Practitioner.name</t>
+  </si>
+  <si>
+    <t>De naamgegevens van de zorgverlener. Indien een zorgverleneridentificatienummer wordt opgegeven, is dit de naam zoals vermeld in UZI, AGB of in de instelling. In het geval dat niet bekend en/of niet relevant is hoe de naamgegevens zijn opgebouwd, kan de subbouwsteen Naamgegevens niet worden gebruikt.</t>
+  </si>
+  <si>
+    <t>ZVL-003</t>
+  </si>
+  <si>
+    <t>Geslacht</t>
+  </si>
+  <si>
+    <t>Practitioner.gender</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Administratief geslacht van de zorgverlener </t>
+  </si>
+  <si>
+    <t>0..1</t>
+  </si>
+  <si>
+    <t>ZVL-004</t>
+  </si>
+  <si>
+    <t>Adresgegevens</t>
+  </si>
+  <si>
+    <t>Practitioner.address</t>
+  </si>
+  <si>
+    <t>Van de zorgverlener</t>
+  </si>
+  <si>
+    <t>Wordt soms niet gedeeld wegens privacy, maar kan bereikt worden via Zorgaanbieder</t>
+  </si>
+  <si>
+    <t>ZVL-005</t>
+  </si>
+  <si>
+    <t>Contactgegevens</t>
+  </si>
+  <si>
+    <t>Practitioner.telecom</t>
+  </si>
+  <si>
+    <t>Telefoonnummer(s) of e-mailadres(sen) van de zorgverlener.</t>
+  </si>
+  <si>
+    <t>Ter Discussie</t>
+  </si>
+  <si>
+    <t>Data element</t>
+  </si>
+  <si>
+    <t>Uitleg</t>
+  </si>
+  <si>
+    <t>Uitkomst</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>Moet DEZI als identifier toegevoegd worden. Niet expliciet genoemd in de zib. Wel al aangekondigd dat het zal worden uitgerold.</t>
+  </si>
+  <si>
+    <t>Wel toegevoegd. In ART-DECOR is er nog geen OID voor. Volgens deze bron wordt gewoon de OID van UZI hergebruikt: https://build.fhir.org/ig/nuts-foundation/nl-generic-functions-ig/credential-DeziUserCredential.html</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
     <t>zib</t>
   </si>
   <si>
-    <t>ZVL-002</t>
-  </si>
-  <si>
-    <t>Naamgegevens</t>
-  </si>
-  <si>
-    <t>Practitioner.name</t>
-  </si>
-  <si>
-    <t>De naamgegevens van de zorgverlener. Indien een zorgverleneridentificatienummer wordt opgegeven, is dit de naam zoals vermeld in UZI, AGB of in de instelling. In het geval dat niet bekend en/of niet relevant is hoe de naamgegevens zijn opgebouwd, kan de subbouwsteen Naamgegevens niet worden gebruikt.</t>
-  </si>
-  <si>
-    <t>ZVL-003</t>
-  </si>
-  <si>
-    <t>Geslacht</t>
-  </si>
-  <si>
-    <t>Practitioner.gender</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Administratief geslacht van de zorgverlener </t>
-  </si>
-  <si>
-    <t>0..1</t>
-  </si>
-  <si>
-    <t>zib2020</t>
-  </si>
-  <si>
-    <t>ZVL-004</t>
-  </si>
-  <si>
-    <t>Adresgegevens</t>
-  </si>
-  <si>
-    <t>Practitioner.address</t>
-  </si>
-  <si>
-    <t>Van de zorgverlener</t>
-  </si>
-  <si>
-    <t>Wordt soms niet gedeeld wegens privacy, maar kan bereikt worden via Zorgaanbieder</t>
-  </si>
-  <si>
-    <t>ZVL-005</t>
-  </si>
-  <si>
-    <t>Contactgegevens</t>
-  </si>
-  <si>
-    <t>Practitioner.telecom</t>
-  </si>
-  <si>
-    <t>Telefoonnummer(s) of e-mailadres(sen) van de zorgverlener.</t>
-  </si>
-  <si>
-    <t>Ter Discussie</t>
-  </si>
-  <si>
-    <t>Data element</t>
-  </si>
-  <si>
-    <t>Uitleg</t>
-  </si>
-  <si>
-    <t>Uitkomst</t>
-  </si>
-  <si>
-    <t>Identifier</t>
-  </si>
-  <si>
-    <t>Moet DEZI als identifier toegevoegd worden. Niet expliciet genoemd in de zib. Wel al aangekondigd dat het zal worden uitgerold.</t>
-  </si>
-  <si>
-    <t>Wel toegevoegd. In ART-DECOR is er nog geen OID voor. Volgens deze bron wordt gewoon de OID van UZI hergebruikt: https://build.fhir.org/ig/nuts-foundation/nl-generic-functions-ig/credential-DeziUserCredential.html</t>
-  </si>
-  <si>
-    <t>gender</t>
-  </si>
-  <si>
     <t>Extensie/waardelijst is overbodig, zie: https://nictiz.atlassian.net/browse/ZIBFHIR-386</t>
   </si>
   <si>
@@ -466,15 +466,6 @@
   </si>
   <si>
     <t>Aanwezigheid</t>
-  </si>
-  <si>
-    <t>Kolom1</t>
-  </si>
-  <si>
-    <t>Kolom2</t>
-  </si>
-  <si>
-    <t>Kolom3</t>
   </si>
   <si>
     <t>[Actie om te ondernemen, kies uit de 3 acties: cluster, andere bouwsteen en modelleren]</t>
@@ -511,19 +502,10 @@
 Het betreft hierbij de erkende medische specialismen zoals vermeld in de wet BIG. Bijvoorbeeld huisarts of cardioloog. </t>
   </si>
   <si>
-    <t>AGB en UZI zijn geprefereerde codesystemen voor nederlandse zorgverleners</t>
-  </si>
-  <si>
-    <t>Richtlijn Verslaglegging</t>
-  </si>
-  <si>
-    <t>e-Overdracht</t>
+    <t>zib-HealthProfessional-v3.5(2020EN)</t>
   </si>
   <si>
     <t>Andere codes dan AGB of UZI(DEZI) specialismecodes</t>
-  </si>
-  <si>
-    <t>Nictiz Sharepoint | Afwijkingenregister eOverdracht</t>
   </si>
   <si>
     <t>PractitionerRole.telecom</t>
@@ -533,9 +515,6 @@
 Telefoonnummer(s) of e-mailadres(sen), kan ook intercollegiaal telefoonnummer</t>
   </si>
   <si>
-    <t>Niet om te delen; communicatie over de overdracht loopt via Zorgdomein (ZE-1)</t>
-  </si>
-  <si>
     <t>Zorgaanbieder</t>
   </si>
   <si>
@@ -554,9 +533,6 @@
     <t>Het concept ZorgverlenerRol kan op twee manieren worden tot uiting worden gebracht, als element in de bouwsteen en als definitiecode bij een verwijzing in een andere bouwsteen (Uitvoerder::Zorgverlener). In beide gevallen wordt voor de code uit dezelfde codelijst geput. Als beide mogelijkheden benut worden, mogen zij niet met elkaar in strijd zijn.</t>
   </si>
   <si>
-    <t>https://www.zibs.nl/images/9/9b/Nl.zorg.Zorgverlener-v3.2%282017NL%29.pdf</t>
-  </si>
-  <si>
     <t>availableTime</t>
   </si>
   <si>
@@ -566,7 +542,7 @@
     <t>Uit zib2020 Contactgegevens.Toelichting (NL-CM:20.6.9) -&gt; "Aangegeven kan bijvoorbeeld worden dat het een afdelingsnummer is (bij zorgverleners) of dat de bereikbaarheid slecht gedurende een aangegeven deel van de dag mogelijk is."</t>
   </si>
   <si>
-    <t>https://zibs.nl/wiki/Contactgegevens-v1.2(2020NL)</t>
+    <t>zib-Contactgegevens-v1.2(2020NL)</t>
   </si>
 </sst>
 </file>
@@ -738,7 +714,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -803,13 +779,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFF1A983"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -875,9 +860,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -909,16 +891,10 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -959,125 +935,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{B0F7F417-6139-AC4A-9919-70BAFABB9069}"/>
   </cellStyles>
-  <dxfs count="38">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FFF1A983"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFF1A983"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFF1A983"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color rgb="FFF1A983"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFF1A983"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color rgb="FFF1A983"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFF1A983"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="35">
     <dxf>
       <font>
         <b val="0"/>
@@ -2055,74 +1932,71 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{6A1F38C1-1851-423E-8C75-57BD38E49F17}" name="Tabel6" displayName="Tabel6" ref="B2:D13" totalsRowShown="0" headerRowBorderDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{6A1F38C1-1851-423E-8C75-57BD38E49F17}" name="Tabel6" displayName="Tabel6" ref="B2:D13" totalsRowShown="0" headerRowBorderDxfId="34">
   <autoFilter ref="B2:D13" xr:uid="{6A1F38C1-1851-423E-8C75-57BD38E49F17}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{9EA81764-1F48-4BA0-AF52-9EDEE7890087}" name="Veld" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{D8142A7B-6921-43C6-8C3F-4A451280F5D7}" name="Beschrijving voorbeeld" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{5AE74986-ACF4-4D7E-A2B4-77152E816BE5}" name="Beschrijving" dataDxfId="34" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{9EA81764-1F48-4BA0-AF52-9EDEE7890087}" name="Veld" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{D8142A7B-6921-43C6-8C3F-4A451280F5D7}" name="Beschrijving voorbeeld" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{5AE74986-ACF4-4D7E-A2B4-77152E816BE5}" name="Beschrijving" dataDxfId="31" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}" name="Tabel4" displayName="Tabel4" ref="B2:D12" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}" name="Tabel4" displayName="Tabel4" ref="B2:D12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
   <autoFilter ref="B2:D12" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B7C9118D-39DF-4758-ADFE-1560AAACC3F5}" name="type bron" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{3978D9DC-65AF-4577-B6A0-E1131DA09C9D}" name="link" dataDxfId="30" dataCellStyle="Hyperlink"/>
-    <tableColumn id="3" xr3:uid="{356ED7AE-934A-47A2-9E12-06B4DD6D8871}" name="aantekeningen" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{B7C9118D-39DF-4758-ADFE-1560AAACC3F5}" name="type bron" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{3978D9DC-65AF-4577-B6A0-E1131DA09C9D}" name="link" dataDxfId="27" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{356ED7AE-934A-47A2-9E12-06B4DD6D8871}" name="aantekeningen" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="B2:J7" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" headerRowBorderDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="B2:J7" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" headerRowBorderDxfId="23">
   <autoFilter ref="B2:J7" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{A7FC29C7-F2D4-48A5-A359-69D6658FB7BA}" name="FHIR data-element" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Voorwaardelijkheid" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Herkomst" dataDxfId="19" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Informatiestandaard" dataDxfId="18" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Vragen" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{A7FC29C7-F2D4-48A5-A359-69D6658FB7BA}" name="FHIR data-element" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Voorwaardelijkheid" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Herkomst" dataDxfId="16" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Informatiestandaard" dataDxfId="15" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Vragen" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E20" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E20" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B3:E20" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}" name="Tabel3" displayName="Tabel3" ref="A1:J8" totalsRowShown="0" headerRowDxfId="10">
-  <autoFilter ref="A1:J8" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{5F814FB7-5678-4579-B8B1-1E5545EDA381}" name="Actie" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{B21F027D-8B76-47A3-924F-04081C8DE379}" name="Notitie" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{E9B0B86A-6F7A-4CA7-80C1-9F863B0F16D2}" name="Naam" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{5370DE7F-F579-4C53-8DC5-4A307EB4AA83}" name="Omschrijving" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{7A38DD6C-13CA-48AF-A56B-A3788AE8DF4A}" name="Variabiliteit" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{DBF2BC9D-E9B3-4CF4-9090-E9489B8EC27C}" name="Aanwezigheid" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{2E747585-23EE-46CF-998B-ED36A36A08C9}" name="Herkomst" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{7F666297-F72F-4181-BD58-84ABD89FE0FF}" name="Kolom1" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{439F2AE8-570D-4AFE-BFD9-62E32720200A}" name="Kolom2" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{F1A4A8F5-082C-42B8-BFB9-E14E0C208A3C}" name="Kolom3" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}" name="Tabel3" displayName="Tabel3" ref="A1:G8" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:G8" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{5F814FB7-5678-4579-B8B1-1E5545EDA381}" name="Actie" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{B21F027D-8B76-47A3-924F-04081C8DE379}" name="Notitie" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{E9B0B86A-6F7A-4CA7-80C1-9F863B0F16D2}" name="Naam" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{5370DE7F-F579-4C53-8DC5-4A307EB4AA83}" name="Omschrijving" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{7A38DD6C-13CA-48AF-A56B-A3788AE8DF4A}" name="Variabiliteit" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{DBF2BC9D-E9B3-4CF4-9090-E9489B8EC27C}" name="Aanwezigheid" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{2E747585-23EE-46CF-998B-ED36A36A08C9}" name="Herkomst" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2470,12 +2344,12 @@
       <c r="C2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="23" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29.25">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="43" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
@@ -2486,7 +2360,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="43.5">
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="43" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="10" t="s">
@@ -2497,7 +2371,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="72.75">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="43" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="10" t="s">
@@ -2508,7 +2382,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="57.75">
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="43" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="10" t="s">
@@ -2519,7 +2393,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="29.25">
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="43" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="10" t="s">
@@ -2530,7 +2404,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="29.25">
-      <c r="B8" s="46" t="s">
+      <c r="B8" s="43" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="10" t="s">
@@ -2541,7 +2415,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="140.25" customHeight="1">
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="43" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="10" t="s">
@@ -2552,11 +2426,11 @@
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="B10" s="47"/>
+      <c r="B10" s="44"/>
       <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:4" ht="43.5">
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="43" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="4" t="s">
@@ -2567,7 +2441,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75">
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="43" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -2579,7 +2453,7 @@
     </row>
     <row r="13" spans="1:4" ht="84" customHeight="1">
       <c r="A13" s="9"/>
-      <c r="B13" s="46" t="s">
+      <c r="B13" s="43" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="10" t="s">
@@ -2617,131 +2491,131 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6">
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="54" t="s">
+      <c r="C2" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="D2" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="40" t="s">
         <v>37</v>
       </c>
       <c r="D3" s="1"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="40" t="s">
         <v>39</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="40" t="s">
         <v>42</v>
       </c>
       <c r="D5" s="1"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="40" t="s">
         <v>44</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="40" t="s">
         <v>46</v>
       </c>
       <c r="D7" s="1"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="43" t="s">
+      <c r="C8" s="40" t="s">
         <v>46</v>
       </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="40" t="s">
         <v>49</v>
       </c>
       <c r="D9" s="1"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="40" t="s">
         <v>51</v>
       </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="43" t="s">
+      <c r="C11" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="41"/>
     </row>
     <row r="12" spans="2:6">
       <c r="B12" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="43" t="s">
+      <c r="C12" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="45"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2768,62 +2642,62 @@
   <dimension ref="A1:L7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="26" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" style="26" customWidth="1"/>
-    <col min="4" max="4" width="31" style="26" customWidth="1"/>
-    <col min="5" max="5" width="65.7109375" style="26" customWidth="1"/>
-    <col min="6" max="6" width="14" style="26" customWidth="1"/>
-    <col min="7" max="7" width="82.7109375" style="27" customWidth="1"/>
-    <col min="8" max="8" width="37.7109375" style="26" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" style="26" customWidth="1"/>
-    <col min="10" max="10" width="35.28515625" style="26" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" style="26" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.85546875" style="26"/>
+    <col min="1" max="1" width="6.140625" style="25" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="31" style="25" customWidth="1"/>
+    <col min="5" max="5" width="65.7109375" style="25" customWidth="1"/>
+    <col min="6" max="6" width="14" style="25" customWidth="1"/>
+    <col min="7" max="7" width="82.7109375" style="26" customWidth="1"/>
+    <col min="8" max="8" width="37.7109375" style="25" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" style="25" customWidth="1"/>
+    <col min="10" max="10" width="35.28515625" style="25" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.85546875" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24" customHeight="1"/>
-    <row r="2" spans="1:12" s="35" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32" t="s">
+    <row r="2" spans="1:12" s="34" customFormat="1" ht="20.25" customHeight="1">
+      <c r="A2" s="30"/>
+      <c r="B2" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="F2" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="33" t="s">
+      <c r="G2" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="33" t="s">
+      <c r="H2" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="I2" s="33" t="s">
+      <c r="I2" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="J2" s="34" t="s">
+      <c r="J2" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
     </row>
     <row r="3" spans="1:12" s="15" customFormat="1" ht="167.25" customHeight="1">
-      <c r="A3" s="29"/>
-      <c r="B3" s="48" t="s">
+      <c r="A3" s="28"/>
+      <c r="B3" s="45" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="49" t="s">
+      <c r="D3" s="46" t="s">
         <v>68</v>
       </c>
       <c r="E3" s="15" t="s">
@@ -2832,28 +2706,28 @@
       <c r="F3" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="47" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="I3" s="47" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="51"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
     </row>
     <row r="4" spans="1:12" s="15" customFormat="1" ht="72.75">
-      <c r="A4" s="29"/>
-      <c r="B4" s="48" t="s">
+      <c r="A4" s="28"/>
+      <c r="B4" s="45" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="49" t="s">
+      <c r="D4" s="46" t="s">
         <v>76</v>
       </c>
       <c r="E4" s="15" t="s">
@@ -2862,26 +2736,26 @@
       <c r="F4" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="50"/>
-      <c r="H4" s="30" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="I4" s="50" t="s">
+      <c r="I4" s="47" t="s">
         <v>73</v>
       </c>
-      <c r="J4" s="51"/>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
     </row>
     <row r="5" spans="1:12" s="15" customFormat="1">
-      <c r="A5" s="28"/>
-      <c r="B5" s="48" t="s">
+      <c r="A5" s="27"/>
+      <c r="B5" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="50" t="s">
+      <c r="C5" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="50" t="s">
+      <c r="D5" s="47" t="s">
         <v>80</v>
       </c>
       <c r="E5" s="15" t="s">
@@ -2890,70 +2764,70 @@
       <c r="F5" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="G5" s="50"/>
-      <c r="H5" s="52" t="s">
+      <c r="G5" s="47"/>
+      <c r="H5" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="I5" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="J5" s="50"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+    </row>
+    <row r="6" spans="1:12" s="15" customFormat="1">
+      <c r="A6" s="27"/>
+      <c r="B6" s="45" t="s">
         <v>83</v>
       </c>
-      <c r="I5" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="J5" s="53"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-    </row>
-    <row r="6" spans="1:12" s="15" customFormat="1">
-      <c r="A6" s="28"/>
-      <c r="B6" s="48" t="s">
+      <c r="C6" s="47" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="D6" s="47" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="50" t="s">
+      <c r="E6" s="15" t="s">
         <v>86</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>87</v>
       </c>
       <c r="F6" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G6" s="50" t="s">
+      <c r="G6" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="I6" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="J6" s="50"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="B7" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="H6" s="52" t="s">
-        <v>83</v>
-      </c>
-      <c r="I6" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="J6" s="53"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="28"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="B7" s="48" t="s">
+      <c r="C7" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="D7" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="E7" t="s">
         <v>91</v>
-      </c>
-      <c r="E7" t="s">
-        <v>92</v>
       </c>
       <c r="F7" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="H7" s="52" t="s">
-        <v>83</v>
-      </c>
-      <c r="I7" s="50" t="s">
+      <c r="H7" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="J7" s="28"/>
+      <c r="I7" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="J7" s="27"/>
     </row>
   </sheetData>
   <phoneticPr fontId="11" type="noConversion"/>
@@ -2986,23 +2860,23 @@
   <sheetData>
     <row r="2" spans="2:8">
       <c r="B2" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D2" s="6"/>
       <c r="F2" s="7"/>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>64</v>
       </c>
       <c r="D3" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="E3" s="21" t="s">
         <v>95</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>96</v>
       </c>
       <c r="F3" s="20"/>
       <c r="G3" s="20"/>
@@ -3010,21 +2884,21 @@
     </row>
     <row r="4" spans="2:8" ht="60">
       <c r="B4" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="E4" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="79.5" customHeight="1">
       <c r="B5" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>73</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>101</v>
@@ -3035,7 +2909,7 @@
     </row>
     <row r="6" spans="2:8" ht="81" customHeight="1">
       <c r="B6" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>103</v>
@@ -3107,7 +2981,7 @@
     </row>
     <row r="13" spans="2:8" ht="29.25">
       <c r="B13" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>115</v>
@@ -3316,250 +3190,231 @@
   <cols>
     <col min="1" max="1" width="17.5703125" style="6" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41" style="6" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="30.85546875" style="6" customWidth="1"/>
     <col min="5" max="5" width="61.7109375" style="6" customWidth="1"/>
-    <col min="6" max="6" width="52.42578125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="6" customWidth="1"/>
     <col min="7" max="7" width="38.7109375" style="6" customWidth="1"/>
-    <col min="8" max="10" width="9.85546875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="25.28515625" style="5" customWidth="1"/>
+    <col min="9" max="10" width="9.85546875" style="5" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" ht="146.25" customHeight="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="C1" s="36" t="s">
+      <c r="C1" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="G1" s="36" t="s">
+      <c r="G1" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="52" t="s">
         <v>122</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="B2" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="C2" s="52" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="90">
-      <c r="A2" s="37" t="s">
+      <c r="D2" s="52" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="E2" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="F2" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="G2" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="E2" s="37" t="s">
+    </row>
+    <row r="3" spans="1:12" s="15" customFormat="1" ht="43.5">
+      <c r="A3" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="B3" s="36"/>
+      <c r="C3" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="37" t="s">
+      <c r="D3" s="37" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" s="15" customFormat="1" ht="60">
-      <c r="A3" s="22" t="s">
+      <c r="E3" s="15" t="s">
         <v>132</v>
-      </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="39" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="39" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>135</v>
       </c>
       <c r="F3" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="39" t="s">
-        <v>136</v>
-      </c>
-      <c r="H3" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="I3" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J3" s="41"/>
+      <c r="G3" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="H3" s="53"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="38"/>
       <c r="K3" s="22"/>
       <c r="L3" s="22"/>
     </row>
-    <row r="4" spans="1:12" s="15" customFormat="1" ht="120">
+    <row r="4" spans="1:12" s="15" customFormat="1">
       <c r="A4" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="39" t="s">
-        <v>133</v>
-      </c>
-      <c r="D4" s="39" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="D4" s="37" t="s">
+        <v>131</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>134</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>139</v>
       </c>
       <c r="F4" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="39"/>
-      <c r="H4" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="I4" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J4" s="41"/>
+      <c r="G4" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="H4" s="53"/>
+      <c r="I4" s="37"/>
+      <c r="J4" s="38"/>
       <c r="K4" s="22"/>
       <c r="L4" s="22"/>
     </row>
     <row r="5" spans="1:12" s="15" customFormat="1" ht="79.5" customHeight="1">
       <c r="A5" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="D5" s="39" t="s">
-        <v>141</v>
+        <v>129</v>
+      </c>
+      <c r="B5" s="36"/>
+      <c r="C5" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" s="37" t="s">
+        <v>135</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F5" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G5" s="39" t="s">
-        <v>143</v>
-      </c>
-      <c r="H5" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="I5" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J5" s="41"/>
+      <c r="G5" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="H5" s="53"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="38"/>
       <c r="K5" s="22"/>
       <c r="L5" s="22"/>
     </row>
-    <row r="6" spans="1:12" s="25" customFormat="1" ht="45">
+    <row r="6" spans="1:12" s="24" customFormat="1">
       <c r="A6" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="39" t="s">
-        <v>144</v>
-      </c>
-      <c r="D6" s="39" t="s">
-        <v>145</v>
+        <v>129</v>
+      </c>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="37" t="s">
+        <v>138</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F6" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="G6" s="39"/>
-      <c r="H6" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="I6" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J6" s="41"/>
+      <c r="G6" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="H6" s="53"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="38"/>
       <c r="K6" s="22"/>
       <c r="L6" s="22"/>
     </row>
-    <row r="7" spans="1:12" s="25" customFormat="1" ht="150">
+    <row r="7" spans="1:12" s="24" customFormat="1" ht="72.75">
       <c r="A7" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" s="38"/>
-      <c r="C7" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="D7" s="39" t="s">
-        <v>148</v>
+        <v>129</v>
+      </c>
+      <c r="B7" s="36"/>
+      <c r="C7" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="D7" s="37" t="s">
+        <v>141</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="F7" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="40" t="s">
-        <v>150</v>
-      </c>
-      <c r="I7" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J7" s="41"/>
+      <c r="G7" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="H7" s="53"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="38"/>
       <c r="K7" s="22"/>
       <c r="L7" s="22"/>
     </row>
-    <row r="8" spans="1:12" s="25" customFormat="1" ht="90">
+    <row r="8" spans="1:12" s="24" customFormat="1" ht="57.75">
       <c r="A8" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="39" t="s">
-        <v>151</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>152</v>
+        <v>129</v>
+      </c>
+      <c r="B8" s="36"/>
+      <c r="C8" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="37" t="s">
+        <v>144</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="F8" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G8" s="39"/>
-      <c r="H8" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="I8" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="J8" s="41"/>
+      <c r="G8" s="55" t="s">
+        <v>146</v>
+      </c>
+      <c r="H8" s="54"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="38"/>
       <c r="K8" s="22"/>
       <c r="L8" s="22"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H8" r:id="rId1" xr:uid="{F4DA18DC-4D73-4DD5-9B2E-09ABCCF87E44}"/>
+    <hyperlink ref="G8" r:id="rId1" xr:uid="{F4DA18DC-4D73-4DD5-9B2E-09ABCCF87E44}"/>
+    <hyperlink ref="G7" r:id="rId2" xr:uid="{D7DEC7D2-07ED-4F56-9D8D-8B70624AE626}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{6C7F8EAA-F0F4-435C-A83B-B6AB080E23A0}"/>
+    <hyperlink ref="G3" r:id="rId4" xr:uid="{B2B41F9E-4D7A-4FED-AD8A-732E4ECF9B33}"/>
+    <hyperlink ref="G5" r:id="rId5" xr:uid="{3AEF2645-A40B-4E9D-AF7B-6F5CFCA0F0CF}"/>
+    <hyperlink ref="G6" r:id="rId6" xr:uid="{C2693D45-1547-478A-B81D-33CAFD97324F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId7"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3586,6 +3441,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3792,23 +3656,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}"/>
 </file>
</xml_diff>

<commit_message>
Practitioner and PractitionerRole: added missing rows in "overzicht" tab
</commit_message>
<xml_diff>
--- a/input/requirements/Practitioner.xlsx
+++ b/input/requirements/Practitioner.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djorai_nict1\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2893DA-4B9D-4C00-A8EF-BF5C7D792DD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE6C0E89-7569-4A8C-8523-F74BA3FEB067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="17" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="134">
   <si>
     <t>Veld</t>
   </si>
@@ -472,6 +472,15 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.4.3.11.60.153.4.16/2026-06-08T00:00:00</t>
+  </si>
+  <si>
+    <t>Afsprakenmodel:</t>
+  </si>
+  <si>
+    <t>Basismodel:</t>
+  </si>
+  <si>
+    <t>ART-DECOR®</t>
   </si>
 </sst>
 </file>
@@ -2256,7 +2265,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C34B65-4906-46E5-852C-E6ACE2E756DA}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -2291,7 +2300,7 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2319,7 +2328,7 @@
       <c r="D7" s="14"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2328,7 +2337,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2359,21 +2368,31 @@
       <c r="B12" s="48"/>
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="48" t="s">
+        <v>133</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B14" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="52" t="s">
+      <c r="B15" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="50"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B14" s="14"/>
-      <c r="C14" s="50"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B15" s="48"/>
       <c r="C15" s="50"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -2381,15 +2400,15 @@
       <c r="C16" s="50"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B17" s="14"/>
+      <c r="B17" s="48"/>
       <c r="C17" s="50"/>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" s="48"/>
+      <c r="B18" s="14"/>
       <c r="C18" s="50"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" s="48"/>
+      <c r="B19" s="14"/>
       <c r="C19" s="50"/>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
@@ -2397,12 +2416,23 @@
       <c r="C20" s="50"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B21" s="14"/>
+      <c r="B21" s="48"/>
       <c r="C21" s="50"/>
     </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B22" s="48"/>
+      <c r="C22" s="50"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B23" s="14"/>
+      <c r="C23" s="50"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B14" r:id="rId1" xr:uid="{CBD438AD-9A25-43B5-B099-648B3338593C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3527,6 +3557,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
@@ -3535,15 +3574,6 @@
     <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3566,6 +3596,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -3580,12 +3618,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add missing pagecontent. Fix concept page
</commit_message>
<xml_diff>
--- a/input/requirements/Practitioner.xlsx
+++ b/input/requirements/Practitioner.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahenket/Development/GitHub/Nictiz/GBB-IG/input/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE6C0E89-7569-4A8C-8523-F74BA3FEB067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764E1B4F-1F44-E244-828D-FFCC1E81BB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="18880" yWindow="-26480" windowWidth="34840" windowHeight="25000" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="17" r:id="rId1"/>
@@ -48,9 +48,9 @@
   <commentList>
     <comment ref="D2" authorId="0" shapeId="0" xr:uid="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Vanuit Xt-EHR alleen naamgegevens 0..1, de rest 0..*</t>
       </text>
     </comment>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="132">
   <si>
     <t>Veld</t>
   </si>
@@ -474,13 +474,7 @@
     <t>2.16.840.1.113883.2.4.3.11.60.153.4.16/2026-06-08T00:00:00</t>
   </si>
   <si>
-    <t>Afsprakenmodel:</t>
-  </si>
-  <si>
     <t>Basismodel:</t>
-  </si>
-  <si>
-    <t>ART-DECOR®</t>
   </si>
 </sst>
 </file>
@@ -830,7 +824,7 @@
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{B0F7F417-6139-AC4A-9919-70BAFABB9069}"/>
   </cellStyles>
   <dxfs count="30">
@@ -2265,17 +2259,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C34B65-4906-46E5-852C-E6ACE2E756DA}">
-  <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="93.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="93.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="190.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="49" t="s">
         <v>0</v>
       </c>
@@ -2283,7 +2277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2291,7 +2285,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2300,7 +2294,7 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="80" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2309,7 +2303,7 @@
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2318,7 +2312,7 @@
       </c>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2328,7 +2322,7 @@
       <c r="D7" s="14"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2337,7 +2331,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="128" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2346,7 +2340,7 @@
       </c>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>119</v>
       </c>
@@ -2355,7 +2349,7 @@
       </c>
       <c r="C10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>121</v>
       </c>
@@ -2364,72 +2358,59 @@
       </c>
       <c r="C11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="48"/>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" s="48" t="s">
+        <v>26</v>
+      </c>
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="80" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>131</v>
-      </c>
-      <c r="B13" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>132</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" ht="216" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="52" t="s">
+      <c r="B13" s="52" t="s">
         <v>16</v>
       </c>
+      <c r="C13" s="50"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B14" s="14"/>
+      <c r="C14" s="50"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B15" s="48"/>
       <c r="C15" s="50"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B16" s="14"/>
       <c r="C16" s="50"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B17" s="48"/>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B17" s="14"/>
       <c r="C17" s="50"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" s="14"/>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B18" s="48"/>
       <c r="C18" s="50"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" s="14"/>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B19" s="48"/>
       <c r="C19" s="50"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" s="48"/>
       <c r="C20" s="50"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B21" s="48"/>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B21" s="14"/>
       <c r="C21" s="50"/>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B22" s="48"/>
-      <c r="C22" s="50"/>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B23" s="14"/>
-      <c r="C23" s="50"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B14" r:id="rId1" xr:uid="{CBD438AD-9A25-43B5-B099-648B3338593C}"/>
+    <hyperlink ref="B12" r:id="rId1" xr:uid="{CBD438AD-9A25-43B5-B099-648B3338593C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
@@ -2439,16 +2420,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D98679E3-F4A5-433B-8B8D-5D68D0E8B75A}">
   <dimension ref="B2:F12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="85.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="44.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="85.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="44.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="29" t="s">
         <v>17</v>
       </c>
@@ -2461,7 +2442,7 @@
       <c r="E2" s="34"/>
       <c r="F2" s="34"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B3" s="8" t="s">
         <v>20</v>
       </c>
@@ -2472,7 +2453,7 @@
       <c r="E3" s="36"/>
       <c r="F3" s="36"/>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B4" s="8" t="s">
         <v>22</v>
       </c>
@@ -2485,7 +2466,7 @@
       <c r="E4" s="36"/>
       <c r="F4" s="36"/>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B5" s="8" t="s">
         <v>25</v>
       </c>
@@ -2496,7 +2477,7 @@
       <c r="E5" s="36"/>
       <c r="F5" s="36"/>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B6" s="8" t="s">
         <v>27</v>
       </c>
@@ -2507,7 +2488,7 @@
       <c r="E6" s="36"/>
       <c r="F6" s="36"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B7" s="8" t="s">
         <v>29</v>
       </c>
@@ -2518,7 +2499,7 @@
       <c r="E7" s="36"/>
       <c r="F7" s="36"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B8" s="8" t="s">
         <v>31</v>
       </c>
@@ -2529,7 +2510,7 @@
       <c r="E8" s="36"/>
       <c r="F8" s="36"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B9" s="8" t="s">
         <v>32</v>
       </c>
@@ -2540,7 +2521,7 @@
       <c r="E9" s="36"/>
       <c r="F9" s="36"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B10" s="8" t="s">
         <v>34</v>
       </c>
@@ -2551,7 +2532,7 @@
       <c r="E10" s="36"/>
       <c r="F10" s="36"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B11" s="8" t="s">
         <v>36</v>
       </c>
@@ -2564,7 +2545,7 @@
       <c r="E11" s="36"/>
       <c r="F11" s="36"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B12" s="8" t="s">
         <v>39</v>
       </c>
@@ -2598,22 +2579,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1A0E3D-BE28-4965-A5FF-C835B3665CFB}">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.88671875" style="20" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" style="20" customWidth="1"/>
     <col min="3" max="3" width="65.6640625" style="20" customWidth="1"/>
     <col min="4" max="4" width="14" style="20" customWidth="1"/>
     <col min="5" max="5" width="82.6640625" style="21" customWidth="1"/>
     <col min="6" max="6" width="37.6640625" style="20" customWidth="1"/>
     <col min="7" max="7" width="20.33203125" style="20" customWidth="1"/>
     <col min="8" max="8" width="35.33203125" style="20" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="20" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="20"/>
+    <col min="9" max="9" width="8.83203125" style="20" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.83203125" style="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:10" s="29" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:10" s="29" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="26" t="s">
         <v>41</v>
       </c>
@@ -2641,7 +2622,7 @@
       <c r="I2" s="25"/>
       <c r="J2" s="25"/>
     </row>
-    <row r="3" spans="1:10" s="11" customFormat="1" ht="167.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" s="11" customFormat="1" ht="167.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="38" t="s">
         <v>47</v>
       </c>
@@ -2665,7 +2646,7 @@
       <c r="I3" s="23"/>
       <c r="J3" s="23"/>
     </row>
-    <row r="4" spans="1:10" s="11" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" s="11" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A4" s="38" t="s">
         <v>52</v>
       </c>
@@ -2687,7 +2668,7 @@
       <c r="I4" s="23"/>
       <c r="J4" s="23"/>
     </row>
-    <row r="5" spans="1:10" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
         <v>54</v>
       </c>
@@ -2709,7 +2690,7 @@
       <c r="I5" s="22"/>
       <c r="J5" s="22"/>
     </row>
-    <row r="6" spans="1:10" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
         <v>57</v>
       </c>
@@ -2733,7 +2714,7 @@
       <c r="I6" s="22"/>
       <c r="J6" s="22"/>
     </row>
-    <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
         <v>61</v>
       </c>
@@ -2765,21 +2746,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920836FF-9BD3-42C9-9F6B-BFE0A0D44840}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" style="5" customWidth="1"/>
+    <col min="1" max="1" width="17.5" style="5" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="30.88671875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.5" style="5" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" style="5" customWidth="1"/>
     <col min="5" max="5" width="61.6640625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.1640625" style="5" customWidth="1"/>
     <col min="7" max="7" width="38.6640625" style="5" customWidth="1"/>
     <col min="8" max="8" width="25.33203125" style="4" customWidth="1"/>
-    <col min="9" max="10" width="9.88671875" style="4" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="4"/>
+    <col min="9" max="10" width="9.83203125" style="4" customWidth="1"/>
+    <col min="11" max="16384" width="9.1640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" ht="146.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="3" customFormat="1" ht="146.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="30" t="s">
         <v>91</v>
       </c>
@@ -2802,7 +2783,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="44" t="s">
         <v>94</v>
       </c>
@@ -2825,7 +2806,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="11" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" s="11" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="18" t="s">
         <v>101</v>
       </c>
@@ -2851,7 +2832,7 @@
       <c r="K3" s="18"/>
       <c r="L3" s="18"/>
     </row>
-    <row r="4" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
         <v>101</v>
       </c>
@@ -2877,7 +2858,7 @@
       <c r="K4" s="18"/>
       <c r="L4" s="18"/>
     </row>
-    <row r="5" spans="1:12" s="11" customFormat="1" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" s="11" customFormat="1" ht="79.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
         <v>101</v>
       </c>
@@ -2903,7 +2884,7 @@
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
     </row>
-    <row r="6" spans="1:12" s="19" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" s="19" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
         <v>101</v>
       </c>
@@ -2929,7 +2910,7 @@
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
     </row>
-    <row r="7" spans="1:12" s="19" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" s="19" customFormat="1" ht="80" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
         <v>101</v>
       </c>
@@ -2955,7 +2936,7 @@
       <c r="K7" s="18"/>
       <c r="L7" s="18"/>
     </row>
-    <row r="8" spans="1:12" s="19" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" s="19" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
         <v>101</v>
       </c>
@@ -3001,7 +2982,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE73AAFD-F820-4002-80EF-0A422C33165C}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3011,27 +2992,27 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E71E66-FD43-4603-91A3-4CCDD6133986}">
   <dimension ref="A2:H64"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.88671875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="3.83203125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.5" style="4" customWidth="1"/>
+    <col min="3" max="3" width="22.5" style="4" customWidth="1"/>
     <col min="4" max="4" width="74" style="4" customWidth="1"/>
     <col min="5" max="5" width="65.33203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="24.44140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="24.5" style="4" customWidth="1"/>
     <col min="7" max="7" width="21.6640625" style="4" customWidth="1"/>
     <col min="8" max="8" width="73.6640625" style="4" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="4"/>
+    <col min="9" max="16384" width="9.1640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D2" s="5"/>
       <c r="F2" s="6"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B3" s="9" t="s">
         <v>65</v>
       </c>
@@ -3048,7 +3029,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" ht="48" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>68</v>
       </c>
@@ -3059,7 +3040,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" ht="79.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
         <v>71</v>
       </c>
@@ -3073,7 +3054,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="81" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="81" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>58</v>
       </c>
@@ -3081,7 +3062,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" ht="78" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>76</v>
       </c>
@@ -3092,7 +3073,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
         <v>44</v>
       </c>
@@ -3104,7 +3085,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B9" s="5" t="s">
         <v>81</v>
       </c>
@@ -3112,7 +3093,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="63.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="5" t="s">
         <v>83</v>
       </c>
@@ -3123,7 +3104,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B11" s="5" t="s">
         <v>86</v>
       </c>
@@ -3134,7 +3115,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
         <v>89</v>
       </c>
@@ -3145,7 +3126,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B13" s="5" t="s">
         <v>68</v>
       </c>
@@ -3156,7 +3137,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B14" s="5" t="s">
         <v>90</v>
       </c>
@@ -3167,178 +3148,178 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B16" s="5"/>
       <c r="D16" s="5"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B17" s="5"/>
       <c r="D17" s="5"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B18" s="5"/>
       <c r="D18" s="5"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B19" s="5"/>
       <c r="D19" s="5"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B20" s="15"/>
       <c r="C20" s="10"/>
       <c r="D20" s="5"/>
     </row>
-    <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="11"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B24" s="5"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B25" s="5"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="5"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="5"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="5"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="5"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="5"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="5"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="5"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="5"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="5"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="5"/>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="5"/>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="5"/>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="5"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="5"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="5"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" s="5"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" s="5"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="5"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" s="5"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="5"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" s="5"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="5"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" s="5"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="5"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="5"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" s="5"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="5"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" s="5"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="5"/>
     </row>
   </sheetData>
@@ -3350,6 +3331,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3556,27 +3557,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3593,29 +3599,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Practitioner: refreshed requirements file
</commit_message>
<xml_diff>
--- a/input/requirements/Practitioner.xlsx
+++ b/input/requirements/Practitioner.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Practitioner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2640" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CDEA821-C0CA-443C-AA04-55A75BC67655}"/>
+  <xr:revisionPtr revIDLastSave="2780" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8962045-9EA3-4E78-B3D1-039E9C67F33B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="655" firstSheet="3" activeTab="2" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="655" firstSheet="2" activeTab="5" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
-    <sheet name="Context" sheetId="3" r:id="rId1"/>
+    <sheet name="Concept" sheetId="17" r:id="rId1"/>
     <sheet name="Bronnen" sheetId="16" r:id="rId2"/>
     <sheet name="Informatiebehoefte" sheetId="12" r:id="rId3"/>
-    <sheet name="Ter discussie" sheetId="2" r:id="rId4"/>
-    <sheet name="Ongedekte informatiebehoefte" sheetId="14" r:id="rId5"/>
-    <sheet name="Overwegingen voor de toekomst" sheetId="15" r:id="rId6"/>
+    <sheet name="Ongedekte informatiebehoefte" sheetId="14" r:id="rId4"/>
+    <sheet name="Overwegingen voor de toekomst" sheetId="15" r:id="rId5"/>
+    <sheet name="Ter discussie" sheetId="2" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,9 +44,11 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={812FD7AE-C33E-4098-9678-0004F1C27ED0}</author>
+    <author>tc={656198AD-16B7-4B38-AF7C-172C35E8DFA0}</author>
+    <author>tc={536E8CB7-D64E-4591-94E5-62B165F057CB}</author>
   </authors>
   <commentList>
-    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -54,44 +56,50 @@
     Vanuit Xt-EHR alleen naamgegevens 0..1, de rest 0..*</t>
       </text>
     </comment>
+    <comment ref="E3" authorId="1" shapeId="0" xr:uid="{656198AD-16B7-4B38-AF7C-172C35E8DFA0}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+[Tasks]
+There is a task anchored to this comment that cannot be viewed in your client.
+Comment:
+    @Daniel Püttmann, kun je hier ook de inhouds-afhankelijke conditie nalopen en wellicht weghalen?</t>
+      </text>
+    </comment>
+    <comment ref="C6" authorId="2" shapeId="0" xr:uid="{536E8CB7-D64E-4591-94E5-62B165F057CB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    kan je deze volledig maken?</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="139">
   <si>
     <t>Veld</t>
   </si>
   <si>
-    <t>Beschrijving voorbeeld</t>
-  </si>
-  <si>
     <t>Beschrijving</t>
   </si>
   <si>
     <t>Conceptbeschrijving</t>
   </si>
   <si>
-    <t>[De definitie of beschrijving van het concept.]</t>
-  </si>
-  <si>
-    <t>Zorgverlener = Gegevens van een natuurlijke persoon die beroepsmatig zorg verleent (NEN7540:2024)</t>
+    <t>Gegevens van een natuurlijke persoon die beroepsmatig zorg verleent (NEN7540:2024)</t>
   </si>
   <si>
     <t>Doel</t>
   </si>
   <si>
-    <t>[De doelen en redenen om het concept vast te leggen en/of uit te wisselen.]</t>
-  </si>
-  <si>
     <t>Het vastleggen en uitwisselen van zorgverlenergegevens. Primair doel is uitwisseling, secundair doel is vastlegging.</t>
   </si>
   <si>
     <t>Gebruiksscenario(’s)</t>
-  </si>
-  <si>
-    <t>[Geeft aan in welke context(en) het concept wordt gebruikt. Geef voorbeelden van gebruik in informatiestandaarden.]</t>
   </si>
   <si>
     <t xml:space="preserve">1. Belangrijk is om te weten wie de hoofdbehandelaar is en hoe met die persoon contact kan worden opgenomen (uit afwijkingenregister eOverdracht, DE-11)
@@ -103,25 +111,16 @@
     <t>Representatie</t>
   </si>
   <si>
-    <t>[Beschrijf hier wat er voor de dossiervorming belangrijk is rondom de levenscyclus en instantiaties van het concept.]</t>
-  </si>
-  <si>
     <t>Het is mogelijk dat de situatie later kan veranderen en daarmee de informatie van het concept</t>
   </si>
   <si>
     <t>Alias(sen)</t>
   </si>
   <si>
-    <t>[Alle bekende synoniemen voor het concept.]</t>
-  </si>
-  <si>
     <t>Zorgprofessional, Behandelaar, Uitvoerder, Aanvrager, Vaststeller, Verzorger</t>
   </si>
   <si>
     <t>Juist gebruik</t>
-  </si>
-  <si>
-    <t>[Beschrijf hier waarvoor het concept WEL bedoeld is.]</t>
   </si>
   <si>
     <t>1. Om verantwoording aan te geven zodat contact kan worden opgezocht over bepaalde bevindingen
@@ -131,62 +130,27 @@
     <t>Onjuist gebruik</t>
   </si>
   <si>
-    <t>[Beschrijf hier waarvoor het concept NIET bedoeld is.]</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Planninginformatie
+    <t>1. Planninginformatie
 2. Informatie over verrichtingen waar een zorgverlener verantwoordelijk voor is: welke verrichtingen heeft die gedaan, welke diagnose heeft die gesteld enz.
 3. Rol van een persoon in de verlening van zorg voor een Patiënt (Uitvoerder, hoofdbehandelaar, enz.)
             De verwachting is dat dit binnen concept "verrichting" wordt vastgelegd
 4. Niet voor personeelbeheer (thuisadres, salarisschaal enz.)
-5. We verwachten geen informatie over een zorgmedewerker (definitie: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>natuurlijke persoon die werkzaamheden verricht of gaat verrichten voor een zorgaanbieder en daarbij patiëntgegevens raadpleegt met behulp van een goedgekeurd inlogmiddel</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <t>Logisch Model</t>
-  </si>
-  <si>
-    <t>[Link naar dataset.]</t>
-  </si>
-  <si>
-    <t>https://decor.nictiz.nl/ad/#/gbb2026bbr-/datasets/dataset/2.16.840.1.113883.2.4.3.11.60.153.1.4/2026-06-08T13:50:54/concept/2.16.840.1.113883.2.4.3.11.60.153.2.1.148/2026-06-08T14:00:05</t>
-  </si>
-  <si>
-    <t>Basis model</t>
-  </si>
-  <si>
-    <t>[Link naar FHIR of OpenEHR model.]</t>
-  </si>
-  <si>
-    <t>https://build.fhir.org/practitioner.html</t>
+5. We verwachten geen informatie over een zorgmedewerker (definitie: natuurlijke persoon die werkzaamheden verricht of gaat verrichten voor een zorgaanbieder en daarbij patiëntgegevens raadpleegt met behulp van een goedgekeurd inlogmiddel)</t>
+  </si>
+  <si>
+    <t>Referenties</t>
+  </si>
+  <si>
+    <t>zie bronnen tabblad</t>
+  </si>
+  <si>
+    <t>ART-DECOR-id</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.16/2026-06-08T00:00:00</t>
   </si>
   <si>
     <t>Beredenering basismodel</t>
-  </si>
-  <si>
-    <t>[Beredenering keuze voor basismodel]</t>
   </si>
   <si>
     <t>1. FHIR is het voornaamste internationale data-uitwisselingsmodel
@@ -235,12 +199,15 @@
     <t>zib-profiel</t>
   </si>
   <si>
-    <t>https://simplifier.net/nictiz-r4-zib2020/~resources?text=healthprofessional&amp;category=Profile</t>
+    <t>https://simplifier.net/nictiz-r4-zib2020/zibhealthprofessionalpractitioner</t>
   </si>
   <si>
     <t>NL-core-R4</t>
   </si>
   <si>
+    <t>https://simplifier.net/nictiz-r4-zib2020/nlcorehealthprofessionalpractitioner</t>
+  </si>
+  <si>
     <t>EU-core-R4</t>
   </si>
   <si>
@@ -250,7 +217,7 @@
     <t>Xt-EHR LIM</t>
   </si>
   <si>
-    <t>https://www.xt-ehr.eu/fhir/models/0.3.0/StructureDefinition-EHDSHealthProfessional.html</t>
+    <t>https://www.xt-ehr.eu/fhir/models/StructureDefinition-EHDSHealthProfessional.html</t>
   </si>
   <si>
     <t>Xt-EHR LIM --&gt; FHIR mapping</t>
@@ -274,34 +241,28 @@
     <t>Naam</t>
   </si>
   <si>
-    <t>FHIR data-element</t>
-  </si>
-  <si>
     <t>Omschrijving</t>
   </si>
   <si>
     <t>Variabiliteit</t>
   </si>
   <si>
-    <t>Voorwaardelijkheid</t>
+    <t>Aanwezigheid</t>
+  </si>
+  <si>
+    <t>Verleden/heden/toekomst</t>
   </si>
   <si>
     <t>Herkomst</t>
   </si>
   <si>
-    <t>Informatiestandaard</t>
-  </si>
-  <si>
-    <t>Vragen</t>
+    <t>Opmerkingen</t>
   </si>
   <si>
     <t>ZVL-001</t>
   </si>
   <si>
-    <t>Identificatienummer</t>
-  </si>
-  <si>
-    <t>Practitioner.identifier</t>
+    <t>Identificatienummer - Practitioner.identifier</t>
   </si>
   <si>
     <t xml:space="preserve">Het zorgverleneridentificatienummer is een nummer dat de zorgverlener uniek identificeert.
@@ -312,169 +273,82 @@
 Voor buitenlandse zorgverleners zijn deze gegevens niet voorhanden. </t>
   </si>
   <si>
+    <t>identifier</t>
+  </si>
+  <si>
+    <t>0..* (Indien een identificatienummer als UZI of AGB nummer wordt meegegeven, moeten naam en nummer overeenkomen.)</t>
+  </si>
+  <si>
+    <t>EHDSPractitioner, zib2020 zorgverlener, Spoedsamenvatting 2.2.0, BgZ-MSZ 2.0</t>
+  </si>
+  <si>
+    <t>ZVL-002</t>
+  </si>
+  <si>
+    <t>Naamgegevens - Practitioner.name</t>
+  </si>
+  <si>
+    <t>De naamgegevens van de zorgverlener. Indien een zorgverleneridentificatienummer wordt opgegeven, is dit de naam zoals vermeld in UZI, AGB of in de instelling. In het geval dat niet bekend en/of niet relevant is hoe de naamgegevens zijn opgebouwd, kan de subbouwsteen Naamgegevens niet worden gebruikt.</t>
+  </si>
+  <si>
+    <t>GBB-HumanName</t>
+  </si>
+  <si>
     <t>0..*</t>
   </si>
   <si>
-    <t>Indien een identificatienummer als UZI of AGB nummer wordt meegegeven, moeten naam en nummer overeenkomen.</t>
-  </si>
-  <si>
-    <t>Zib 2020</t>
-  </si>
-  <si>
-    <t>zib</t>
-  </si>
-  <si>
-    <t>ZVL-002</t>
-  </si>
-  <si>
-    <t>Naamgegevens</t>
-  </si>
-  <si>
-    <t>Practitioner.name</t>
-  </si>
-  <si>
-    <t>De naamgegevens van de zorgverlener. Indien een zorgverleneridentificatienummer wordt opgegeven, is dit de naam zoals vermeld in UZI, AGB of in de instelling. In het geval dat niet bekend en/of niet relevant is hoe de naamgegevens zijn opgebouwd, kan de subbouwsteen Naamgegevens niet worden gebruikt.</t>
-  </si>
-  <si>
     <t>ZVL-003</t>
   </si>
   <si>
-    <t>Geslacht</t>
-  </si>
-  <si>
-    <t>Practitioner.gender</t>
+    <t>Geslacht - Practitioner.gender</t>
   </si>
   <si>
     <t xml:space="preserve"> Administratief geslacht van de zorgverlener </t>
   </si>
   <si>
+    <t>coded</t>
+  </si>
+  <si>
     <t>0..1</t>
   </si>
   <si>
-    <t>zib2020</t>
+    <t>zib2020 zorgverlener</t>
+  </si>
+  <si>
+    <t>LET OP: dit gaat over aanhef, zie ZIB-1142. Mogelijk te vervangen door pronouns, prefix/suffix (titles)</t>
   </si>
   <si>
     <t>ZVL-004</t>
   </si>
   <si>
-    <t>Adresgegevens</t>
-  </si>
-  <si>
-    <t>Practitioner.address</t>
-  </si>
-  <si>
-    <t>Van de zorgverlener</t>
-  </si>
-  <si>
-    <t>Wordt soms niet gedeeld wegens privacy, maar kan bereikt worden via Zorgaanbieder</t>
+    <t>Adresgegevens - Practitioner.address</t>
+  </si>
+  <si>
+    <t>Rol-agnostisch adresinformatie van een zorgverlener (meestal Thuisadres)</t>
+  </si>
+  <si>
+    <t>GBB-Adress</t>
+  </si>
+  <si>
+    <t>0..* (Wordt soms niet gedeeld wegens privacy, maar kan bereikt worden via Zorgaanbieder of ZorgverlenerRol)</t>
   </si>
   <si>
     <t>ZVL-005</t>
   </si>
   <si>
-    <t>Contactgegevens</t>
-  </si>
-  <si>
-    <t>Practitioner.telecom</t>
+    <t>Contactgegevens - Practitioner.telecom</t>
   </si>
   <si>
     <t>Telefoonnummer(s) of e-mailadres(sen) van de zorgverlener.</t>
   </si>
   <si>
-    <t>Ter Discussie</t>
-  </si>
-  <si>
-    <t>Data element</t>
-  </si>
-  <si>
-    <t>Uitleg</t>
-  </si>
-  <si>
-    <t>Uitkomst</t>
-  </si>
-  <si>
-    <t>Identifier</t>
-  </si>
-  <si>
-    <t>Moet DEZI als identifier toegevoegd worden. Niet expliciet genoemd in de zib. Wel al aangekondigd dat het zal worden uitgerold.</t>
-  </si>
-  <si>
-    <t>Wel toegevoegd. In ART-DECOR is er nog geen OID voor. Volgens deze bron wordt gewoon de OID van UZI hergebruikt: https://build.fhir.org/ig/nuts-foundation/nl-generic-functions-ig/credential-DeziUserCredential.html</t>
-  </si>
-  <si>
-    <t>gender</t>
-  </si>
-  <si>
-    <t>Extensie/waardelijst is overbodig, zie: https://nictiz.atlassian.net/browse/ZIBFHIR-386</t>
-  </si>
-  <si>
-    <t>FHIR waardelijst is gebruikt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In veel gevallen/ aantal standaarden worden er geen adresgegevens van zorgverleners vastgelegd of wel afgeleid uit de zorgaanbieder. Uitzondering kan zijn adresgegevens van huisarts/eigen praktijk. </t>
-  </si>
-  <si>
-    <t>ProfessionalRole</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In de Xt-EHR Health Professional LIM is ook PractitionerRole (role, organization, specialty) onderdeel van het model. </t>
-  </si>
-  <si>
-    <t>Nu wij werken met basismodellen, en dit lostrekken, van elkaar wordt dit onderdeel bekeken vanuit het basismodel PractitionerRole</t>
-  </si>
-  <si>
-    <t>Hoe geven we variabiliteit aan vanuit verschillende bronnen</t>
-  </si>
-  <si>
-    <t>Meenemen als nieuwe requirement indien nog niet gedekt</t>
-  </si>
-  <si>
-    <t>PractitionerName</t>
-  </si>
-  <si>
-    <t>In profiel card. 0..*, wijzigen naar 0..1? Xt-EHR ook 0..1</t>
-  </si>
-  <si>
-    <t>Context container</t>
-  </si>
-  <si>
-    <t>In basismodel komt het vaker voor dat een element van een bijzonder datatype is, bijv. element Name van het datatype HumanName. Hoe wordt de modellering in A-D? Rechtreeks een verwijzing naar HumanName of modelleren als ContextContainer Name met daarin een verwijzing naar HumanName? Dit is waarschijnlijk alleen een A-D probleem en wordt opgelost als we FHIR IG's gebruiken (zoals Xt-EHR)</t>
-  </si>
-  <si>
-    <t>Pro: Met contextcontainer kan verduidelijkt worden welke HumanName of wel ContactPoint wordt bedoeld. Dit geldt ook voor verwijzingen naar andere bouwstenen. Con: Meer gelaagdheid maakt model complexer, en wellicht opgelost door FHIR IG</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>In Xt-EHR wordt dit gemapt op zowel Practioner als PractitionerRole</t>
-  </si>
-  <si>
-    <t>Alleen Telecom meegenomen in afsprakenmodel PractitionerRole, in lijn met nlcore</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Telecom</t>
+    <t>GBB-ContactPoint</t>
   </si>
   <si>
     <t>Actie</t>
   </si>
   <si>
     <t>Notitie</t>
-  </si>
-  <si>
-    <t>Aanwezigheid</t>
-  </si>
-  <si>
-    <t>Kolom1</t>
-  </si>
-  <si>
-    <t>Kolom2</t>
-  </si>
-  <si>
-    <t>Kolom3</t>
   </si>
   <si>
     <t>[Actie om te ondernemen, kies uit de 3 acties: cluster, andere bouwsteen en modelleren]</t>
@@ -511,19 +385,13 @@
 Het betreft hierbij de erkende medische specialismen zoals vermeld in de wet BIG. Bijvoorbeeld huisarts of cardioloog. </t>
   </si>
   <si>
-    <t>AGB en UZI zijn geprefereerde codesystemen voor nederlandse zorgverleners</t>
-  </si>
-  <si>
-    <t>Richtlijn Verslaglegging</t>
-  </si>
-  <si>
-    <t>e-Overdracht</t>
+    <t>zib-HealthProfessional-v3.5(2020EN)</t>
   </si>
   <si>
     <t>Andere codes dan AGB of UZI(DEZI) specialismecodes</t>
   </si>
   <si>
-    <t>Nictiz Sharepoint | Afwijkingenregister eOverdracht</t>
+    <t>Contactgegevens</t>
   </si>
   <si>
     <t>PractitionerRole.telecom</t>
@@ -533,9 +401,6 @@
 Telefoonnummer(s) of e-mailadres(sen), kan ook intercollegiaal telefoonnummer</t>
   </si>
   <si>
-    <t>Niet om te delen; communicatie over de overdracht loopt via Zorgdomein (ZE-1)</t>
-  </si>
-  <si>
     <t>Zorgaanbieder</t>
   </si>
   <si>
@@ -554,9 +419,6 @@
     <t>Het concept ZorgverlenerRol kan op twee manieren worden tot uiting worden gebracht, als element in de bouwsteen en als definitiecode bij een verwijzing in een andere bouwsteen (Uitvoerder::Zorgverlener). In beide gevallen wordt voor de code uit dezelfde codelijst geput. Als beide mogelijkheden benut worden, mogen zij niet met elkaar in strijd zijn.</t>
   </si>
   <si>
-    <t>https://www.zibs.nl/images/9/9b/Nl.zorg.Zorgverlener-v3.2%282017NL%29.pdf</t>
-  </si>
-  <si>
     <t>availableTime</t>
   </si>
   <si>
@@ -566,14 +428,101 @@
     <t>Uit zib2020 Contactgegevens.Toelichting (NL-CM:20.6.9) -&gt; "Aangegeven kan bijvoorbeeld worden dat het een afdelingsnummer is (bij zorgverleners) of dat de bereikbaarheid slecht gedurende een aangegeven deel van de dag mogelijk is."</t>
   </si>
   <si>
-    <t>https://zibs.nl/wiki/Contactgegevens-v1.2(2020NL)</t>
+    <t>zib-Contactgegevens-v1.2(2020NL)</t>
+  </si>
+  <si>
+    <t>Ter Discussie</t>
+  </si>
+  <si>
+    <t>Data element</t>
+  </si>
+  <si>
+    <t>Informatiestandaard</t>
+  </si>
+  <si>
+    <t>Uitleg</t>
+  </si>
+  <si>
+    <t>Uitkomst</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>Moet DEZI als identifier toegevoegd worden. Niet expliciet genoemd in de zib. Wel al aangekondigd dat het zal worden uitgerold.</t>
+  </si>
+  <si>
+    <t>Wel toegevoegd. In ART-DECOR is er nog geen OID voor. Volgens deze bron wordt gewoon de OID van UZI hergebruikt: https://build.fhir.org/ig/nuts-foundation/nl-generic-functions-ig/credential-DeziUserCredential.html</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>zib</t>
+  </si>
+  <si>
+    <t>Extensie/waardelijst is overbodig, zie: https://nictiz.atlassian.net/browse/ZIBFHIR-386</t>
+  </si>
+  <si>
+    <t>FHIR waardelijst is gebruikt</t>
+  </si>
+  <si>
+    <t>Adresgegevens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In veel gevallen/ aantal standaarden worden er geen adresgegevens van zorgverleners vastgelegd of wel afgeleid uit de zorgaanbieder. Uitzondering kan zijn adresgegevens van huisarts/eigen praktijk. </t>
+  </si>
+  <si>
+    <t>ProfessionalRole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In de Xt-EHR Health Professional LIM is ook PractitionerRole (role, organization, specialty) onderdeel van het model. </t>
+  </si>
+  <si>
+    <t>Nu wij werken met basismodellen, en dit lostrekken, van elkaar wordt dit onderdeel bekeken vanuit het basismodel PractitionerRole</t>
+  </si>
+  <si>
+    <t>Hoe geven we variabiliteit aan vanuit verschillende bronnen</t>
+  </si>
+  <si>
+    <t>Meenemen als nieuwe requirement indien nog niet gedekt</t>
+  </si>
+  <si>
+    <t>PractitionerName</t>
+  </si>
+  <si>
+    <t>In profiel card. 0..*, wijzigen naar 0..1? Xt-EHR ook 0..1</t>
+  </si>
+  <si>
+    <t>Context container</t>
+  </si>
+  <si>
+    <t>In basismodel komt het vaker voor dat een element van een bijzonder datatype is, bijv. element Name van het datatype HumanName. Hoe wordt de modellering in A-D? Rechtreeks een verwijzing naar HumanName of modelleren als ContextContainer Name met daarin een verwijzing naar HumanName? Dit is waarschijnlijk alleen een A-D probleem en wordt opgelost als we FHIR IG's gebruiken (zoals Xt-EHR)</t>
+  </si>
+  <si>
+    <t>Pro: Met contextcontainer kan verduidelijkt worden welke HumanName of wel ContactPoint wordt bedoeld. Dit geldt ook voor verwijzingen naar andere bouwstenen. Con: Meer gelaagdheid maakt model complexer, en wellicht opgelost door FHIR IG</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>In Xt-EHR wordt dit gemapt op zowel Practioner als PractitionerRole</t>
+  </si>
+  <si>
+    <t>Alleen Telecom meegenomen in afsprakenmodel PractitionerRole, in lijn met nlcore</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Telecom</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -603,40 +552,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="2" tint="-0.499984740745262"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="2" tint="-0.499984740745262"/>
-      <name val="Aptos"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -711,8 +626,14 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -731,12 +652,6 @@
         <bgColor rgb="FFE97132"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -744,15 +659,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -803,13 +709,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFF1A983"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -820,9 +735,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -832,19 +744,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -853,10 +756,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -868,58 +771,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -932,77 +800,106 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{B0F7F417-6139-AC4A-9919-70BAFABB9069}"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="34">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FFF1A983"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFF1A983"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFF1A983"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1016,66 +913,27 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color auto="1"/>
+        <color theme="0"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
-        <scheme val="none"/>
+        <scheme val="minor"/>
       </font>
       <fill>
-        <patternFill patternType="none">
+        <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor theme="5"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color rgb="FFF1A983"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFF1A983"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color rgb="FFF1A983"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFF1A983"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -1311,79 +1169,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </left>
-        <right style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -1400,7 +1185,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1459,7 +1244,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1500,28 +1285,6 @@
           <fgColor indexed="64"/>
           <bgColor auto="1"/>
         </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none"/>
       </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1566,7 +1329,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1592,7 +1355,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1617,7 +1380,7 @@
           <bgColor rgb="FFE97132"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -1683,26 +1446,13 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="2" tint="-0.499984740745262"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top"/>
     </dxf>
     <dxf>
       <font>
@@ -1715,26 +1465,13 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="12"/>
+        <sz val="11"/>
         <color theme="1"/>
-        <name val="Aptos"/>
+        <name val="Aptos Narrow"/>
         <family val="2"/>
-        <scheme val="none"/>
+        <scheme val="minor"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
+      <alignment horizontal="left" vertical="top"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1754,7 +1491,188 @@
 </styleSheet>
 </file>
 
+<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
+  <Task id="{3C7671F0-5638-4B67-B2DC-2E949DF0AF40}">
+    <Anchor>
+      <Comment id="{656198AD-16B7-4B38-AF7C-172C35E8DFA0}"/>
+    </Anchor>
+    <History>
+      <Event time="2026-07-03T09:41:01.83" id="{2D9D1E80-8B3E-49DE-B49C-7DB4928547E2}">
+        <Attribution userId="S::taco.spitters@nictiz.nl::eff47e48-8544-4500-97c8-7e55e3c068e7" userName="Taco Spitters" userProvider="AD"/>
+        <Anchor>
+          <Comment id="{656198AD-16B7-4B38-AF7C-172C35E8DFA0}"/>
+        </Anchor>
+        <Create/>
+      </Event>
+      <Event time="2026-07-03T09:41:01.83" id="{089CE6FD-FBD3-4672-8A50-461C1AAE70F1}">
+        <Attribution userId="S::taco.spitters@nictiz.nl::eff47e48-8544-4500-97c8-7e55e3c068e7" userName="Taco Spitters" userProvider="AD"/>
+        <Anchor>
+          <Comment id="{656198AD-16B7-4B38-AF7C-172C35E8DFA0}"/>
+        </Anchor>
+        <Assign userId="S::daniel.puttmann@nictiz.nl::b79205a6-7857-4254-a32a-2da36179b3ef" userName="Daniel Püttmann" userProvider="AD"/>
+      </Event>
+      <Event time="2026-07-03T09:41:01.83" id="{D2F983F2-D3BD-48C9-B82D-7580478A4D59}">
+        <Attribution userId="S::taco.spitters@nictiz.nl::eff47e48-8544-4500-97c8-7e55e3c068e7" userName="Taco Spitters" userProvider="AD"/>
+        <Anchor>
+          <Comment id="{656198AD-16B7-4B38-AF7C-172C35E8DFA0}"/>
+        </Anchor>
+        <SetTitle title="@Daniel Püttmann, kun je hier ook de inhouds-afhankelijke conditie nalopen en wellicht weghalen?"/>
+      </Event>
+    </History>
+  </Task>
+</Tasks>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>223837</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>2181225</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94510223-F3AD-49CE-895B-E3B867187516}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="163830" y="221932"/>
+          <a:ext cx="6808470" cy="1961198"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Elk concept wordt geïntroduceerd met een tabel die:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr lvl="0"/>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Het klinische concept identificeert dat door het concept wordt weergegeven, en</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="nl-NL" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr lvl="0"/>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>De belangrijkste kenmerken beschrijft die relevant zijn voor de implementatie, inclusief het beoogde gebruik en veelvoorkomende fouten in gebruik.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Deze tabel is bedoeld om een aantal standaard checkvragen te beantwoorden. Deze antwoorden zullen doorgaans blijken uit de informatiebehoefte die onder paragraaf 1.3 beschreven wordt (het is dus niet zo dat eerst de tabel wordt ingevuld en daarna pas de informatiebehoefte).</a:t>
+          </a:r>
+          <a:endParaRPr lang="nl-NL" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1999,7 +1917,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2050,79 +1968,76 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Daniel Püttmann" id="{6865BC61-9325-483B-A60C-7A2937038FDA}" userId="daniel.puttmann@nictiz.nl" providerId="PeoplePicker"/>
+  <person displayName="Taco Spitters" id="{0219CB87-FB9F-48A3-9223-580539FD96F0}" userId="S::taco.spitters@nictiz.nl::eff47e48-8544-4500-97c8-7e55e3c068e7" providerId="AD"/>
   <person displayName="Micha Drielinger" id="{1324D2D7-870F-4779-B1C5-13BE7166ED9A}" userId="S::micha.drielinger@nictiz.nl::240cb811-65d1-423b-aaca-0429a1ee5686" providerId="AD"/>
 </personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{6A1F38C1-1851-423E-8C75-57BD38E49F17}" name="Tabel6" displayName="Tabel6" ref="B2:D13" totalsRowShown="0" headerRowBorderDxfId="37">
-  <autoFilter ref="B2:D13" xr:uid="{6A1F38C1-1851-423E-8C75-57BD38E49F17}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{9EA81764-1F48-4BA0-AF52-9EDEE7890087}" name="Veld" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{D8142A7B-6921-43C6-8C3F-4A451280F5D7}" name="Beschrijving voorbeeld" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{5AE74986-ACF4-4D7E-A2B4-77152E816BE5}" name="Beschrijving" dataDxfId="34" dataCellStyle="Hyperlink"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1A79D11A-83AE-4F16-9DD7-93E839755155}" name="Tabel5" displayName="Tabel5" ref="A2:B12" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+  <autoFilter ref="A2:B12" xr:uid="{1A79D11A-83AE-4F16-9DD7-93E839755155}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{D6F958DF-C12C-4ABF-BBA5-B7387AA5194D}" name="Veld" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{F824B42B-A1A9-4D9E-8ED7-09B1A44B0BBB}" name="Beschrijving" dataDxfId="30" dataCellStyle="Standaard 2"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}" name="Tabel4" displayName="Tabel4" ref="B2:D12" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}" name="Tabel4" displayName="Tabel4" ref="B2:D12" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="B2:D12" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B7C9118D-39DF-4758-ADFE-1560AAACC3F5}" name="type bron" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{3978D9DC-65AF-4577-B6A0-E1131DA09C9D}" name="link" dataDxfId="30" dataCellStyle="Hyperlink"/>
-    <tableColumn id="3" xr3:uid="{356ED7AE-934A-47A2-9E12-06B4DD6D8871}" name="aantekeningen" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{B7C9118D-39DF-4758-ADFE-1560AAACC3F5}" name="type bron" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{3978D9DC-65AF-4577-B6A0-E1131DA09C9D}" name="link" dataDxfId="26" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{356ED7AE-934A-47A2-9E12-06B4DD6D8871}" name="aantekeningen" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="B2:J7" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" headerRowBorderDxfId="26">
-  <autoFilter ref="B2:J7" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{A7FC29C7-F2D4-48A5-A359-69D6658FB7BA}" name="FHIR data-element" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Voorwaardelijkheid" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Herkomst" dataDxfId="19" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Informatiestandaard" dataDxfId="18" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Vragen" dataDxfId="17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:H7" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23" headerRowBorderDxfId="22">
+  <autoFilter ref="A2:H7" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="16" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="15" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E20" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
-  <autoFilter ref="B3:E20" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}" name="Tabel3" displayName="Tabel3" ref="A1:G8" totalsRowShown="0" headerRowDxfId="13">
+  <autoFilter ref="A1:G8" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{5F814FB7-5678-4579-B8B1-1E5545EDA381}" name="Actie" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{B21F027D-8B76-47A3-924F-04081C8DE379}" name="Notitie" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{E9B0B86A-6F7A-4CA7-80C1-9F863B0F16D2}" name="Naam" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{5370DE7F-F579-4C53-8DC5-4A307EB4AA83}" name="Omschrijving" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{7A38DD6C-13CA-48AF-A56B-A3788AE8DF4A}" name="Variabiliteit" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{DBF2BC9D-E9B3-4CF4-9090-E9489B8EC27C}" name="Aanwezigheid" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{2E747585-23EE-46CF-998B-ED36A36A08C9}" name="Herkomst" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}" name="Tabel3" displayName="Tabel3" ref="A1:J8" totalsRowShown="0" headerRowDxfId="10">
-  <autoFilter ref="A1:J8" xr:uid="{8F51AAA4-3F83-4CED-B767-3181BDCF6575}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{5F814FB7-5678-4579-B8B1-1E5545EDA381}" name="Actie" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{B21F027D-8B76-47A3-924F-04081C8DE379}" name="Notitie" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{E9B0B86A-6F7A-4CA7-80C1-9F863B0F16D2}" name="Naam" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{5370DE7F-F579-4C53-8DC5-4A307EB4AA83}" name="Omschrijving" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{7A38DD6C-13CA-48AF-A56B-A3788AE8DF4A}" name="Variabiliteit" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{DBF2BC9D-E9B3-4CF4-9090-E9489B8EC27C}" name="Aanwezigheid" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{2E747585-23EE-46CF-998B-ED36A36A08C9}" name="Herkomst" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{7F666297-F72F-4181-BD58-84ABD89FE0FF}" name="Kolom1" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{439F2AE8-570D-4AFE-BFD9-62E32720200A}" name="Kolom2" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{F1A4A8F5-082C-42B8-BFB9-E14E0C208A3C}" name="Kolom3" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E20" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="B3:E20" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2445,161 +2360,171 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F2" dT="2026-06-10T07:13:12.83" personId="{1324D2D7-870F-4779-B1C5-13BE7166ED9A}" id="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
+  <threadedComment ref="D2" dT="2026-06-10T07:13:12.83" personId="{1324D2D7-870F-4779-B1C5-13BE7166ED9A}" id="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
     <text>Vanuit Xt-EHR alleen naamgegevens 0..1, de rest 0..*</text>
+  </threadedComment>
+  <threadedComment ref="E3" dT="2026-07-03T09:41:01.97" personId="{0219CB87-FB9F-48A3-9223-580539FD96F0}" id="{656198AD-16B7-4B38-AF7C-172C35E8DFA0}">
+    <text>@Daniel Püttmann, kun je hier ook de inhouds-afhankelijke conditie nalopen en wellicht weghalen?</text>
+    <mentions>
+      <mention mentionpersonId="{6865BC61-9325-483B-A60C-7A2937038FDA}" mentionId="{664BF9D6-346A-40D7-A8DC-79AA229A3CA7}" startIndex="0" length="16"/>
+    </mentions>
+  </threadedComment>
+  <threadedComment ref="C6" dT="2026-07-03T09:43:28.41" personId="{0219CB87-FB9F-48A3-9223-580539FD96F0}" id="{536E8CB7-D64E-4591-94E5-62B165F057CB}" done="1">
+    <text>kan je deze volledig maken?</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44D01FA7-4587-470D-A390-D8587FD365B7}">
-  <dimension ref="A2:D14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C34B65-4906-46E5-852C-E6ACE2E756DA}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="28.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="97" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="140.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" ht="15.75">
-      <c r="B2" s="8" t="s">
+    <row r="1" spans="1:5" ht="190.5" customHeight="1">
+      <c r="A1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="15">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="24" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="15">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="29.25">
       <c r="B3" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="10" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="15">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B4" s="46" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="43.5">
-      <c r="B4" s="46" t="s">
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" ht="57.75">
+      <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="B5" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" ht="15">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="72.75">
-      <c r="B5" s="46" t="s">
+      <c r="B6" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" ht="15">
+      <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="B7" s="46" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="57.75">
-      <c r="B6" s="46" t="s">
+      <c r="D7" s="14"/>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" ht="29.25">
+      <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="B8" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" ht="109.5" customHeight="1">
+      <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="29.25">
-      <c r="B7" s="46" t="s">
+      <c r="B9" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" ht="15">
+      <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="B10" s="46" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="29.25">
-      <c r="B8" s="46" t="s">
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" ht="15">
+      <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="B11" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" ht="77.25" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="140.25" customHeight="1">
-      <c r="B9" s="46" t="s">
+      <c r="B12" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="B10" s="47"/>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" ht="43.5">
-      <c r="B11" s="46" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75">
-      <c r="B12" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="84" customHeight="1">
-      <c r="A13" s="9"/>
-      <c r="B13" s="46" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="9"/>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" ht="15">
+      <c r="C13" s="35"/>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="B14" s="14"/>
+      <c r="C14" s="35"/>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="B15" s="34"/>
+      <c r="C15" s="35"/>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="B16" s="14"/>
+      <c r="C16" s="35"/>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="14"/>
+      <c r="C17" s="35"/>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="34"/>
+      <c r="C18" s="35"/>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="34"/>
+      <c r="C19" s="35"/>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="34"/>
+      <c r="C20" s="35"/>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" s="14"/>
+      <c r="C21" s="35"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D12" r:id="rId1" xr:uid="{C5DAE231-8FBC-455F-AFB2-5A8C5FD666CE}"/>
-    <hyperlink ref="D11" r:id="rId2" location="/gbb2026bbr-/datasets/dataset/2.16.840.1.113883.2.4.3.11.60.153.1.4/2026-06-08T13:50:54/concept/2.16.840.1.113883.2.4.3.11.60.153.2.1.148/2026-06-08T14:00:05" xr:uid="{ED889409-A698-4A14-A40D-FE70B64C7857}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2607,7 +2532,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D98679E3-F4A5-433B-8B8D-5D68D0E8B75A}">
   <dimension ref="B2:F12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -2617,131 +2542,131 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6">
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+    </row>
+    <row r="3" spans="2:6">
+      <c r="B3" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+    </row>
+    <row r="4" spans="2:6">
+      <c r="B4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+    </row>
+    <row r="5" spans="2:6">
+      <c r="B5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+    </row>
+    <row r="6" spans="2:6">
+      <c r="B6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="54" t="s">
+      <c r="D6" s="1"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+    </row>
+    <row r="7" spans="2:6" ht="15">
+      <c r="B7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="C7" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-    </row>
-    <row r="3" spans="2:6">
-      <c r="B3" s="12" t="s">
+      <c r="D7" s="1"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+    </row>
+    <row r="8" spans="2:6" ht="15">
+      <c r="B8" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C8" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-    </row>
-    <row r="4" spans="2:6">
-      <c r="B4" s="12" t="s">
+      <c r="D8" s="1"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+    </row>
+    <row r="9" spans="2:6">
+      <c r="B9" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C9" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D9" s="1"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+    </row>
+    <row r="10" spans="2:6" ht="15">
+      <c r="B10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-    </row>
-    <row r="5" spans="2:6">
-      <c r="B5" s="12" t="s">
+      <c r="C10" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="D10" s="1"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+    </row>
+    <row r="11" spans="2:6">
+      <c r="B11" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-    </row>
-    <row r="6" spans="2:6">
-      <c r="B6" s="12" t="s">
+      <c r="C11" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="D11" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-    </row>
-    <row r="7" spans="2:6">
-      <c r="B7" s="12" t="s">
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+    </row>
+    <row r="12" spans="2:6">
+      <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C12" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-    </row>
-    <row r="8" spans="2:6">
-      <c r="B8" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="43" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-    </row>
-    <row r="9" spans="2:6">
-      <c r="B9" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-    </row>
-    <row r="10" spans="2:6">
-      <c r="B10" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-    </row>
-    <row r="11" spans="2:6">
-      <c r="B11" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="43" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="45" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-    </row>
-    <row r="12" spans="2:6">
-      <c r="B12" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="43" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="45"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2765,541 +2690,758 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1A0E3D-BE28-4965-A5FF-C835B3665CFB}">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="26" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" style="26" customWidth="1"/>
-    <col min="4" max="4" width="31" style="26" customWidth="1"/>
-    <col min="5" max="5" width="65.7109375" style="26" customWidth="1"/>
-    <col min="6" max="6" width="14" style="26" customWidth="1"/>
-    <col min="7" max="7" width="82.7109375" style="27" customWidth="1"/>
-    <col min="8" max="8" width="37.7109375" style="26" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" style="26" customWidth="1"/>
-    <col min="10" max="10" width="35.28515625" style="26" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" style="26" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.85546875" style="26"/>
+    <col min="1" max="1" width="10.42578125" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="65.7109375" style="11" customWidth="1"/>
+    <col min="4" max="4" width="14" style="11" customWidth="1"/>
+    <col min="5" max="5" width="82.7109375" style="11" customWidth="1"/>
+    <col min="6" max="6" width="37.7109375" style="11" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="33.7109375" style="11" customWidth="1"/>
+    <col min="8" max="8" width="35.28515625" style="11" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="24" customHeight="1"/>
-    <row r="2" spans="1:12" s="35" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32" t="s">
+    <row r="1" spans="1:10" ht="24" customHeight="1"/>
+    <row r="2" spans="1:10" s="15" customFormat="1" ht="20.25" customHeight="1">
+      <c r="A2" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="43" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+    </row>
+    <row r="3" spans="1:10" ht="167.25" customHeight="1">
+      <c r="A3" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="D3" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="E3" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="F3" s="38"/>
+      <c r="G3" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="H3" s="39"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+    </row>
+    <row r="4" spans="1:10" ht="72.75">
+      <c r="A4" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="33" t="s">
+      <c r="B4" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="33" t="s">
+      <c r="C4" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="I2" s="33" t="s">
+      <c r="D4" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="J2" s="34" t="s">
+      <c r="E4" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-    </row>
-    <row r="3" spans="1:12" s="15" customFormat="1" ht="167.25" customHeight="1">
-      <c r="A3" s="29"/>
-      <c r="B3" s="48" t="s">
+      <c r="F4" s="38"/>
+      <c r="G4" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" s="39"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+    </row>
+    <row r="5" spans="1:10" ht="43.5">
+      <c r="A5" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="49" t="s">
+      <c r="B5" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="49" t="s">
+      <c r="C5" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="D5" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="E5" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="F5" s="41"/>
+      <c r="G5" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H5" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
+    </row>
+    <row r="6" spans="1:10" ht="43.5">
+      <c r="A6" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="51"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-    </row>
-    <row r="4" spans="1:12" s="15" customFormat="1" ht="72.75">
-      <c r="A4" s="29"/>
-      <c r="B4" s="48" t="s">
+      <c r="B6" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C6" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="49" t="s">
+      <c r="D6" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E6" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G4" s="50"/>
-      <c r="H4" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="I4" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="J4" s="51"/>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
-    </row>
-    <row r="5" spans="1:12" s="15" customFormat="1">
-      <c r="A5" s="28"/>
-      <c r="B5" s="48" t="s">
+      <c r="F6" s="41"/>
+      <c r="G6" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H6" s="39"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
+    </row>
+    <row r="7" spans="1:10" ht="43.5">
+      <c r="A7" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="50" t="s">
+      <c r="B7" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="50" t="s">
+      <c r="C7" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="D7" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="F5" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="G5" s="50"/>
-      <c r="H5" s="52" t="s">
-        <v>83</v>
-      </c>
-      <c r="I5" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="J5" s="53"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-    </row>
-    <row r="6" spans="1:12" s="15" customFormat="1">
-      <c r="A6" s="28"/>
-      <c r="B6" s="48" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="50" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G6" s="50" t="s">
-        <v>88</v>
-      </c>
-      <c r="H6" s="52" t="s">
-        <v>83</v>
-      </c>
-      <c r="I6" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="J6" s="53"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="28"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="B7" s="48" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="E7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="H7" s="52" t="s">
-        <v>83</v>
-      </c>
-      <c r="I7" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="J7" s="28"/>
+      <c r="E7" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="41"/>
+      <c r="G7" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" s="40"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="11" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="H4" r:id="rId1" xr:uid="{5934E9FF-9271-40F1-8E8B-10E4A4A9BE75}"/>
-  </hyperlinks>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920836FF-9BD3-42C9-9F6B-BFE0A0D44840}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="30.85546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="61.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="38.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="25.28515625" style="4" customWidth="1"/>
+    <col min="9" max="10" width="9.85546875" style="4" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="3" customFormat="1" ht="146.25" customHeight="1">
+      <c r="A1" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" s="11" customFormat="1" ht="43.15">
+      <c r="A3" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="22"/>
+      <c r="C3" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="H3" s="31"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+    </row>
+    <row r="4" spans="1:12" s="11" customFormat="1">
+      <c r="A4" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="31"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+    </row>
+    <row r="5" spans="1:12" s="11" customFormat="1" ht="79.5" customHeight="1">
+      <c r="A5" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="22"/>
+      <c r="C5" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="H5" s="31"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+    </row>
+    <row r="6" spans="1:12" s="19" customFormat="1" ht="15">
+      <c r="A6" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="22"/>
+      <c r="C6" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="H6" s="31"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+    </row>
+    <row r="7" spans="1:12" s="19" customFormat="1" ht="72">
+      <c r="A7" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="H7" s="31"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+    </row>
+    <row r="8" spans="1:12" s="19" customFormat="1" ht="57.6">
+      <c r="A8" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="22"/>
+      <c r="C8" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="H8" s="32"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G8" r:id="rId1" xr:uid="{F4DA18DC-4D73-4DD5-9B2E-09ABCCF87E44}"/>
+    <hyperlink ref="G7" r:id="rId2" xr:uid="{D7DEC7D2-07ED-4F56-9D8D-8B70624AE626}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{6C7F8EAA-F0F4-435C-A83B-B6AB080E23A0}"/>
+    <hyperlink ref="G3" r:id="rId4" xr:uid="{B2B41F9E-4D7A-4FED-AD8A-732E4ECF9B33}"/>
+    <hyperlink ref="G5" r:id="rId5" xr:uid="{3AEF2645-A40B-4E9D-AF7B-6F5CFCA0F0CF}"/>
+    <hyperlink ref="G6" r:id="rId6" xr:uid="{C2693D45-1547-478A-B81D-33CAFD97324F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId7"/>
+  <tableParts count="1">
+    <tablePart r:id="rId8"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE73AAFD-F820-4002-80EF-0A422C33165C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E71E66-FD43-4603-91A3-4CCDD6133986}">
   <dimension ref="A2:H64"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="3.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="74" style="5" customWidth="1"/>
-    <col min="5" max="5" width="65.28515625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="24.42578125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="73.7109375" style="5" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="3.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="74" style="4" customWidth="1"/>
+    <col min="5" max="5" width="65.28515625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="24.42578125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="73.7109375" style="4" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8">
-      <c r="B2" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="D2" s="6"/>
-      <c r="F2" s="7"/>
+      <c r="B2" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="3" spans="2:8">
-      <c r="B3" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-    </row>
-    <row r="4" spans="2:8" ht="60">
-      <c r="B4" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>99</v>
+      <c r="B3" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+    </row>
+    <row r="4" spans="2:8" ht="43.15">
+      <c r="B4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="79.5" customHeight="1">
-      <c r="B5" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>102</v>
+      <c r="B5" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="81" customHeight="1">
-      <c r="B6" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>103</v>
+      <c r="B6" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="78" customHeight="1">
-      <c r="B7" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>105</v>
+      <c r="B7" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="2:8">
-      <c r="B8" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>108</v>
+      <c r="B8" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>110</v>
+      <c r="B9" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="63.75" customHeight="1">
-      <c r="B10" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" ht="29.25">
-      <c r="B11" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="B10" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="28.9">
+      <c r="B11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" ht="28.9">
+      <c r="B12" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" ht="28.9">
+      <c r="B13" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" ht="29.25">
-      <c r="B12" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" ht="29.25">
-      <c r="B13" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" ht="29.25">
-      <c r="B14" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>116</v>
+      <c r="D13" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="28.9">
+      <c r="B14" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="2:8">
-      <c r="B15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="B15" s="5"/>
+      <c r="D15" s="5"/>
     </row>
     <row r="16" spans="2:8">
-      <c r="B16" s="6"/>
-      <c r="D16" s="6"/>
+      <c r="B16" s="5"/>
+      <c r="D16" s="5"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="B17" s="6"/>
-      <c r="D17" s="6"/>
+      <c r="B17" s="5"/>
+      <c r="D17" s="5"/>
     </row>
     <row r="18" spans="1:4">
-      <c r="B18" s="6"/>
-      <c r="D18" s="6"/>
+      <c r="B18" s="5"/>
+      <c r="D18" s="5"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="B19" s="6"/>
-      <c r="D19" s="6"/>
+      <c r="B19" s="5"/>
+      <c r="D19" s="5"/>
     </row>
     <row r="20" spans="1:4">
-      <c r="B20" s="19"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="6"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="5"/>
     </row>
     <row r="21" spans="1:4" ht="19.5" customHeight="1">
-      <c r="B21" s="15"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
     </row>
     <row r="22" spans="1:4" ht="19.5" customHeight="1">
-      <c r="B22" s="15"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
     </row>
     <row r="23" spans="1:4" ht="19.5" customHeight="1">
-      <c r="B23" s="6"/>
+      <c r="B23" s="5"/>
     </row>
     <row r="24" spans="1:4">
-      <c r="B24" s="6"/>
+      <c r="B24" s="5"/>
     </row>
     <row r="25" spans="1:4">
-      <c r="B25" s="6"/>
+      <c r="B25" s="5"/>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="6"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6"/>
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="6"/>
-      <c r="B28" s="6"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="6"/>
-      <c r="B29" s="6"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6"/>
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="6"/>
-      <c r="B32" s="6"/>
+      <c r="A32" s="5"/>
+      <c r="B32" s="5"/>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="6"/>
-      <c r="B35" s="6"/>
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="6"/>
+      <c r="A37" s="5"/>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="6"/>
+      <c r="A38" s="5"/>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="6"/>
+      <c r="A39" s="5"/>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="6"/>
+      <c r="A40" s="5"/>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="6"/>
+      <c r="A41" s="5"/>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="6"/>
+      <c r="A42" s="5"/>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="6"/>
+      <c r="A43" s="5"/>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="6"/>
+      <c r="A44" s="5"/>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="6"/>
+      <c r="A45" s="5"/>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="6"/>
+      <c r="A46" s="5"/>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="6"/>
+      <c r="A47" s="5"/>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="6"/>
+      <c r="A48" s="5"/>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="6"/>
+      <c r="A49" s="5"/>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" s="6"/>
+      <c r="A50" s="5"/>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="6"/>
+      <c r="A51" s="5"/>
     </row>
     <row r="52" spans="1:1">
-      <c r="A52" s="6"/>
+      <c r="A52" s="5"/>
     </row>
     <row r="53" spans="1:1">
-      <c r="A53" s="6"/>
+      <c r="A53" s="5"/>
     </row>
     <row r="54" spans="1:1">
-      <c r="A54" s="6"/>
+      <c r="A54" s="5"/>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" s="6"/>
+      <c r="A55" s="5"/>
     </row>
     <row r="56" spans="1:1">
-      <c r="A56" s="6"/>
+      <c r="A56" s="5"/>
     </row>
     <row r="57" spans="1:1">
-      <c r="A57" s="6"/>
+      <c r="A57" s="5"/>
     </row>
     <row r="58" spans="1:1">
-      <c r="A58" s="6"/>
+      <c r="A58" s="5"/>
     </row>
     <row r="59" spans="1:1">
-      <c r="A59" s="6"/>
+      <c r="A59" s="5"/>
     </row>
     <row r="60" spans="1:1">
-      <c r="A60" s="6"/>
+      <c r="A60" s="5"/>
     </row>
     <row r="61" spans="1:1">
-      <c r="A61" s="6"/>
+      <c r="A61" s="5"/>
     </row>
     <row r="62" spans="1:1">
-      <c r="A62" s="6"/>
+      <c r="A62" s="5"/>
     </row>
     <row r="63" spans="1:1">
-      <c r="A63" s="6"/>
+      <c r="A63" s="5"/>
     </row>
     <row r="64" spans="1:1">
-      <c r="A64" s="6"/>
+      <c r="A64" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3309,272 +3451,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920836FF-9BD3-42C9-9F6B-BFE0A0D44840}">
-  <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="17.5703125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41" style="6" customWidth="1"/>
-    <col min="5" max="5" width="61.7109375" style="6" customWidth="1"/>
-    <col min="6" max="6" width="52.42578125" style="6" customWidth="1"/>
-    <col min="7" max="7" width="38.7109375" style="6" customWidth="1"/>
-    <col min="8" max="10" width="9.85546875" style="5" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" ht="146.25" customHeight="1">
-      <c r="A1" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="C1" s="36" t="s">
-        <v>58</v>
-      </c>
-      <c r="D1" s="36" t="s">
-        <v>60</v>
-      </c>
-      <c r="E1" s="36" t="s">
-        <v>61</v>
-      </c>
-      <c r="F1" s="36" t="s">
-        <v>121</v>
-      </c>
-      <c r="G1" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="90">
-      <c r="A2" s="37" t="s">
-        <v>125</v>
-      </c>
-      <c r="B2" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="C2" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>128</v>
-      </c>
-      <c r="E2" s="37" t="s">
-        <v>129</v>
-      </c>
-      <c r="F2" s="37" t="s">
-        <v>130</v>
-      </c>
-      <c r="G2" s="37" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" s="15" customFormat="1" ht="60">
-      <c r="A3" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="39" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="39" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G3" s="39" t="s">
-        <v>136</v>
-      </c>
-      <c r="H3" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="I3" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J3" s="41"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-    </row>
-    <row r="4" spans="1:12" s="15" customFormat="1" ht="120">
-      <c r="A4" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="39" t="s">
-        <v>133</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>134</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G4" s="39"/>
-      <c r="H4" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="I4" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J4" s="41"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-    </row>
-    <row r="5" spans="1:12" s="15" customFormat="1" ht="79.5" customHeight="1">
-      <c r="A5" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="D5" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G5" s="39" t="s">
-        <v>143</v>
-      </c>
-      <c r="H5" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="I5" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J5" s="41"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-    </row>
-    <row r="6" spans="1:12" s="25" customFormat="1" ht="45">
-      <c r="A6" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="39" t="s">
-        <v>144</v>
-      </c>
-      <c r="D6" s="39" t="s">
-        <v>145</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="G6" s="39"/>
-      <c r="H6" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="I6" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J6" s="41"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-    </row>
-    <row r="7" spans="1:12" s="25" customFormat="1" ht="150">
-      <c r="A7" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" s="38"/>
-      <c r="C7" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="D7" s="39" t="s">
-        <v>148</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="40" t="s">
-        <v>150</v>
-      </c>
-      <c r="I7" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="J7" s="41"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-    </row>
-    <row r="8" spans="1:12" s="25" customFormat="1" ht="90">
-      <c r="A8" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="39" t="s">
-        <v>151</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>152</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G8" s="39"/>
-      <c r="H8" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="I8" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="J8" s="41"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="H8" r:id="rId1" xr:uid="{F4DA18DC-4D73-4DD5-9B2E-09ABCCF87E44}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
-  </tableParts>
-</worksheet>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE73AAFD-F820-4002-80EF-0A422C33165C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
@@ -3585,7 +3471,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3792,23 +3678,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
 </file>
</xml_diff>

<commit_message>
Practitioner: added EU filter row
</commit_message>
<xml_diff>
--- a/input/requirements/Practitioner.xlsx
+++ b/input/requirements/Practitioner.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Practitioner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2780" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8962045-9EA3-4E78-B3D1-039E9C67F33B}"/>
+  <xr:revisionPtr revIDLastSave="2783" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93AD6C00-2DFF-41BC-92AC-1BFABCEC36DA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="655" firstSheet="2" activeTab="5" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="655" firstSheet="5" activeTab="2" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="17" r:id="rId1"/>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="140">
   <si>
     <t>Veld</t>
   </si>
@@ -257,6 +257,9 @@
   </si>
   <si>
     <t>Opmerkingen</t>
+  </si>
+  <si>
+    <t>EU filter</t>
   </si>
   <si>
     <t>ZVL-001</t>
@@ -653,7 +656,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -718,13 +721,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFF1A983"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFF1A983"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFF1A983"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFF1A983"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -819,33 +855,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -855,14 +867,41 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{B0F7F417-6139-AC4A-9919-70BAFABB9069}"/>
   </cellStyles>
-  <dxfs count="34">
+  <dxfs count="35">
     <dxf>
       <fill>
         <patternFill patternType="none"/>
@@ -1167,6 +1206,26 @@
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1975,40 +2034,43 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1A79D11A-83AE-4F16-9DD7-93E839755155}" name="Tabel5" displayName="Tabel5" ref="A2:B12" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1A79D11A-83AE-4F16-9DD7-93E839755155}" name="Tabel5" displayName="Tabel5" ref="A2:B12" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="A2:B12" xr:uid="{1A79D11A-83AE-4F16-9DD7-93E839755155}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D6F958DF-C12C-4ABF-BBA5-B7387AA5194D}" name="Veld" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{F824B42B-A1A9-4D9E-8ED7-09B1A44B0BBB}" name="Beschrijving" dataDxfId="30" dataCellStyle="Standaard 2"/>
+    <tableColumn id="1" xr3:uid="{D6F958DF-C12C-4ABF-BBA5-B7387AA5194D}" name="Veld" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{F824B42B-A1A9-4D9E-8ED7-09B1A44B0BBB}" name="Beschrijving" dataDxfId="31" dataCellStyle="Standaard 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}" name="Tabel4" displayName="Tabel4" ref="B2:D12" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}" name="Tabel4" displayName="Tabel4" ref="B2:D12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
   <autoFilter ref="B2:D12" xr:uid="{AABA32E5-8DAE-4C72-8504-E228F7E1A3B2}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B7C9118D-39DF-4758-ADFE-1560AAACC3F5}" name="type bron" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{3978D9DC-65AF-4577-B6A0-E1131DA09C9D}" name="link" dataDxfId="26" dataCellStyle="Hyperlink"/>
-    <tableColumn id="3" xr3:uid="{356ED7AE-934A-47A2-9E12-06B4DD6D8871}" name="aantekeningen" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{B7C9118D-39DF-4758-ADFE-1560AAACC3F5}" name="type bron" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{3978D9DC-65AF-4577-B6A0-E1131DA09C9D}" name="link" dataDxfId="27" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{356ED7AE-934A-47A2-9E12-06B4DD6D8871}" name="aantekeningen" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:H7" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23" headerRowBorderDxfId="22">
-  <autoFilter ref="A2:H7" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="16" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="15" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:I7" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" headerRowBorderDxfId="23">
+  <autoFilter ref="A2:I7" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="17" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="16" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{A82999A8-5F5D-4DC9-84DE-0D99871FB0E8}" name="EU filter" dataDxfId="14">
+      <calculatedColumnFormula>ISNUMBER(SEARCH("EHDS", G3))</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2399,7 +2461,7 @@
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="38" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2407,7 +2469,7 @@
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="38" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="2"/>
@@ -2416,7 +2478,7 @@
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="39" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="2"/>
@@ -2425,7 +2487,7 @@
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="38" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="2"/>
@@ -2434,7 +2496,7 @@
       <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="38" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="14"/>
@@ -2444,7 +2506,7 @@
       <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="47" t="s">
+      <c r="B8" s="39" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="2"/>
@@ -2453,7 +2515,7 @@
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="47" t="s">
+      <c r="B9" s="39" t="s">
         <v>15</v>
       </c>
       <c r="C9" s="2"/>
@@ -2462,7 +2524,7 @@
       <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="46" t="s">
+      <c r="B10" s="38" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="2"/>
@@ -2471,7 +2533,7 @@
       <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="40" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="2"/>
@@ -2480,7 +2542,7 @@
       <c r="A12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="47" t="s">
+      <c r="B12" s="39" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="2"/>
@@ -2707,152 +2769,170 @@
   <sheetData>
     <row r="1" spans="1:10" ht="24" customHeight="1"/>
     <row r="2" spans="1:10" s="15" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="43" t="s">
+      <c r="E2" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="43" t="s">
+      <c r="F2" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="43" t="s">
+      <c r="G2" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="44" t="s">
+      <c r="H2" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
+      <c r="I2" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="J2" s="37"/>
     </row>
     <row r="3" spans="1:10" ht="167.25" customHeight="1">
-      <c r="A3" s="36" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="37" t="s">
+      <c r="A3" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="B3" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="C3" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="D3" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="F3" s="38"/>
-      <c r="G3" s="37" t="s">
+      <c r="E3" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="39"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42" t="b">
+        <f t="shared" ref="I3:I7" si="0">ISNUMBER(SEARCH("EHDS", G3))</f>
+        <v>1</v>
+      </c>
+      <c r="J3" s="36"/>
     </row>
     <row r="4" spans="1:10" ht="72.75">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="42" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="47" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" s="47" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" s="41"/>
+      <c r="G4" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="F4" s="38"/>
-      <c r="G4" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="H4" s="39"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J4" s="36"/>
     </row>
     <row r="5" spans="1:10" ht="43.5">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="47" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" s="48"/>
+      <c r="G5" s="42" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" s="42" t="s">
+        <v>73</v>
+      </c>
+      <c r="I5" s="42" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J5" s="36"/>
+    </row>
+    <row r="6" spans="1:10" ht="43.5">
+      <c r="A6" s="42" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="42" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="47" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="47" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" s="48"/>
+      <c r="G6" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J6" s="36"/>
+    </row>
+    <row r="7" spans="1:10" ht="43.5">
+      <c r="A7" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="47" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="E7" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="37" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="F5" s="41"/>
-      <c r="G5" s="37" t="s">
-        <v>71</v>
-      </c>
-      <c r="H5" s="39" t="s">
-        <v>72</v>
-      </c>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
-    </row>
-    <row r="6" spans="1:10" ht="43.5">
-      <c r="A6" s="36" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="F6" s="41"/>
-      <c r="G6" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="39"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="40"/>
-    </row>
-    <row r="7" spans="1:10" ht="43.5">
-      <c r="A7" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="41"/>
-      <c r="G7" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="H7" s="40"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -2883,10 +2963,10 @@
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" ht="146.25" customHeight="1">
       <c r="A1" s="21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C1" s="21" t="s">
         <v>48</v>
@@ -2906,46 +2986,46 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G2" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:12" s="11" customFormat="1" ht="43.15">
       <c r="A3" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B3" s="22"/>
       <c r="C3" s="23" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H3" s="31"/>
       <c r="I3" s="23"/>
@@ -2955,23 +3035,23 @@
     </row>
     <row r="4" spans="1:12" s="11" customFormat="1">
       <c r="A4" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="23" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E4" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" s="34" t="s">
         <v>96</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" s="34" t="s">
-        <v>95</v>
       </c>
       <c r="H4" s="31"/>
       <c r="I4" s="23"/>
@@ -2981,23 +3061,23 @@
     </row>
     <row r="5" spans="1:12" s="11" customFormat="1" ht="79.5" customHeight="1">
       <c r="A5" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="22"/>
       <c r="C5" s="23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H5" s="31"/>
       <c r="I5" s="23"/>
@@ -3007,23 +3087,23 @@
     </row>
     <row r="6" spans="1:12" s="19" customFormat="1" ht="15">
       <c r="A6" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G6" s="34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H6" s="31"/>
       <c r="I6" s="23"/>
@@ -3033,23 +3113,23 @@
     </row>
     <row r="7" spans="1:12" s="19" customFormat="1" ht="72">
       <c r="A7" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H7" s="31"/>
       <c r="I7" s="23"/>
@@ -3059,23 +3139,23 @@
     </row>
     <row r="8" spans="1:12" s="19" customFormat="1" ht="57.6">
       <c r="A8" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B8" s="22"/>
       <c r="C8" s="23" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G8" s="33" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H8" s="32"/>
       <c r="I8" s="23"/>
@@ -3128,23 +3208,23 @@
   <sheetData>
     <row r="2" spans="2:8">
       <c r="B2" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D2" s="5"/>
       <c r="F2" s="6"/>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F3" s="16"/>
       <c r="G3" s="16"/>
@@ -3152,46 +3232,46 @@
     </row>
     <row r="4" spans="2:8" ht="43.15">
       <c r="B4" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="79.5" customHeight="1">
       <c r="B5" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="81" customHeight="1">
       <c r="B6" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="78" customHeight="1">
       <c r="B7" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="2:8">
@@ -3200,73 +3280,73 @@
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="2:8">
       <c r="B9" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="63.75" customHeight="1">
       <c r="B10" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="28.9">
       <c r="B11" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="28.9">
       <c r="B12" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="28.9">
       <c r="B13" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="28.9">
       <c r="B14" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="2:8">
@@ -3452,15 +3532,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
@@ -3469,6 +3540,15 @@
     <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3679,11 +3759,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>